<commit_message>
Actualizacion al formato de requeriminetos de cambios
</commit_message>
<xml_diff>
--- a/Documentacion/12 Matriz de Gestion de Calidad.xlsx
+++ b/Documentacion/12 Matriz de Gestion de Calidad.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBBFE41-AAB5-4D1B-ACB8-1AD1896D642D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -1707,31 +1707,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1759,7 +1738,28 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -3075,7 +3075,7 @@
     <row r="1" spans="1:17" ht="25.05" customHeight="1">
       <c r="A1" s="12"/>
       <c r="B1" s="12"/>
-      <c r="C1" s="43" t="s">
+      <c r="C1" s="58" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="42"/>
@@ -3115,58 +3115,58 @@
       <c r="Q2" s="44"/>
     </row>
     <row r="3" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="59" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46" t="s">
+      <c r="B3" s="60"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46" t="s">
+      <c r="F3" s="60"/>
+      <c r="G3" s="60"/>
+      <c r="H3" s="60"/>
+      <c r="I3" s="60" t="s">
         <v>84</v>
       </c>
-      <c r="J3" s="46"/>
-      <c r="K3" s="46"/>
-      <c r="L3" s="46"/>
-      <c r="M3" s="46" t="s">
+      <c r="J3" s="60"/>
+      <c r="K3" s="60"/>
+      <c r="L3" s="60"/>
+      <c r="M3" s="60" t="s">
         <v>85</v>
       </c>
-      <c r="N3" s="46"/>
-      <c r="O3" s="46"/>
-      <c r="P3" s="46"/>
-      <c r="Q3" s="47"/>
+      <c r="N3" s="60"/>
+      <c r="O3" s="60"/>
+      <c r="P3" s="60"/>
+      <c r="Q3" s="61"/>
     </row>
     <row r="4" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="54" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49" t="s">
+      <c r="B4" s="55"/>
+      <c r="C4" s="55"/>
+      <c r="D4" s="55"/>
+      <c r="E4" s="55" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="49"/>
-      <c r="G4" s="49"/>
-      <c r="H4" s="49"/>
-      <c r="I4" s="49" t="s">
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
+      <c r="H4" s="55"/>
+      <c r="I4" s="55" t="s">
         <v>88</v>
       </c>
-      <c r="J4" s="49"/>
-      <c r="K4" s="49"/>
-      <c r="L4" s="49"/>
-      <c r="M4" s="49" t="s">
+      <c r="J4" s="55"/>
+      <c r="K4" s="55"/>
+      <c r="L4" s="55"/>
+      <c r="M4" s="55" t="s">
         <v>89</v>
       </c>
-      <c r="N4" s="49"/>
-      <c r="O4" s="49"/>
-      <c r="P4" s="49"/>
-      <c r="Q4" s="50"/>
+      <c r="N4" s="55"/>
+      <c r="O4" s="55"/>
+      <c r="P4" s="55"/>
+      <c r="Q4" s="56"/>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="13"/>
@@ -3188,7 +3188,7 @@
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="24" customHeight="1">
-      <c r="A6" s="51" t="s">
+      <c r="A6" s="57" t="s">
         <v>90</v>
       </c>
       <c r="B6" s="44"/>
@@ -3209,94 +3209,94 @@
       <c r="Q6" s="44"/>
     </row>
     <row r="7" spans="1:17" ht="24" customHeight="1">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="52"/>
+      <c r="B7" s="45"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="52" t="s">
+      <c r="D7" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="52"/>
+      <c r="E7" s="45"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="52" t="s">
+      <c r="G7" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="52"/>
+      <c r="H7" s="45"/>
       <c r="I7" s="14"/>
-      <c r="J7" s="52" t="s">
+      <c r="J7" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="52"/>
+      <c r="K7" s="45"/>
       <c r="L7" s="14"/>
-      <c r="M7" s="52" t="s">
+      <c r="M7" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="N7" s="52"/>
+      <c r="N7" s="45"/>
       <c r="O7" s="14"/>
-      <c r="P7" s="52" t="s">
+      <c r="P7" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="Q7" s="52"/>
+      <c r="Q7" s="45"/>
     </row>
     <row r="8" spans="1:17" ht="24" customHeight="1">
-      <c r="A8" s="53">
+      <c r="A8" s="46">
         <f>COUNTA(A13:A76)</f>
         <v>64</v>
       </c>
-      <c r="B8" s="54"/>
+      <c r="B8" s="47"/>
       <c r="C8" s="15"/>
-      <c r="D8" s="54">
+      <c r="D8" s="47">
         <f>COUNTIF(I13:I76,"Cumple")+COUNTIF(I13:I76,"Cumple parcialmente")+COUNTIF(I13:I76,"No cumple")+COUNTIF(I13:I76,"No aplica")</f>
         <v>2</v>
       </c>
-      <c r="E8" s="54"/>
+      <c r="E8" s="47"/>
       <c r="F8" s="15"/>
-      <c r="G8" s="57">
+      <c r="G8" s="50">
         <f>IFERROR(D8/A8,0)</f>
         <v>3.125E-2</v>
       </c>
-      <c r="H8" s="57"/>
+      <c r="H8" s="50"/>
       <c r="I8" s="15"/>
-      <c r="J8" s="57">
+      <c r="J8" s="50">
         <f>IFERROR(SUM(J13:J76)/(COUNT(J13:J76)*2),0)</f>
         <v>1</v>
       </c>
-      <c r="K8" s="57"/>
+      <c r="K8" s="50"/>
       <c r="L8" s="15"/>
-      <c r="M8" s="57">
+      <c r="M8" s="50">
         <f>IFERROR(COUNTIF(I13:I76,"Cumple")/COUNT(J13:J76),0)</f>
         <v>1</v>
       </c>
-      <c r="N8" s="57"/>
+      <c r="N8" s="50"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="54" t="str">
+      <c r="P8" s="47" t="str">
         <f>IF(G8&lt;1,"PENDIENTE DE EVALUACIÓN",IF(COUNTIFS(G13:G76,"Highest",I13:I76,"No cumple")&gt;0,"NO APROBADO",IF(J8&gt;=0.9,"APROBADO","REQUIERE MEJORAS")))</f>
         <v>PENDIENTE DE EVALUACIÓN</v>
       </c>
-      <c r="Q8" s="59"/>
+      <c r="Q8" s="52"/>
     </row>
     <row r="9" spans="1:17" ht="24" customHeight="1">
-      <c r="A9" s="55"/>
-      <c r="B9" s="56"/>
+      <c r="A9" s="48"/>
+      <c r="B9" s="49"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="56"/>
-      <c r="E9" s="56"/>
+      <c r="D9" s="49"/>
+      <c r="E9" s="49"/>
       <c r="F9" s="16"/>
-      <c r="G9" s="58"/>
-      <c r="H9" s="58"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="58"/>
-      <c r="K9" s="58"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
       <c r="L9" s="16"/>
-      <c r="M9" s="58"/>
-      <c r="N9" s="58"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
       <c r="O9" s="16"/>
-      <c r="P9" s="56"/>
-      <c r="Q9" s="60"/>
+      <c r="P9" s="49"/>
+      <c r="Q9" s="53"/>
     </row>
     <row r="10" spans="1:17" ht="24" customHeight="1">
-      <c r="A10" s="61" t="s">
+      <c r="A10" s="43" t="s">
         <v>92</v>
       </c>
       <c r="B10" s="44"/>
@@ -5807,6 +5807,17 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C1:Q1"/>
+    <mergeCell ref="C2:Q2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="I4:L4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="A6:Q6"/>
     <mergeCell ref="A10:Q10"/>
     <mergeCell ref="P7:Q7"/>
     <mergeCell ref="A8:B9"/>
@@ -5820,17 +5831,6 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="I4:L4"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="C1:Q1"/>
-    <mergeCell ref="C2:Q2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="M3:Q3"/>
   </mergeCells>
   <conditionalFormatting sqref="G13:G76">
     <cfRule type="cellIs" dxfId="12" priority="5" operator="equal">

</xml_diff>

<commit_message>
Actualizacion de Control de Cambios
</commit_message>
<xml_diff>
--- a/Documentacion/12 Matriz de Gestion de Calidad.xlsx
+++ b/Documentacion/12 Matriz de Gestion de Calidad.xlsx
@@ -5,17 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\U Alex\Ingenieria Software 2\Proyecto Ingenieria II\Documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexMendoza\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EBBFE41-AAB5-4D1B-ACB8-1AD1896D642D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCD307D-9169-497F-A23E-64F55BC33354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
     <sheet name="Matriz de calidad" sheetId="2" r:id="rId2"/>
     <sheet name="Catálogos" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="Métricas de calidad" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="481">
   <si>
     <t>BARRIO SOLIDARIO</t>
   </si>
@@ -286,15 +287,9 @@
     <t>Código: DOC-08</t>
   </si>
   <si>
-    <t>Versión: 1.0.0</t>
-  </si>
-  <si>
     <t>Estado: En elaboración</t>
   </si>
   <si>
-    <t>Actualización: 14/09/2026</t>
-  </si>
-  <si>
     <t>Propietario: Luis Rodríguez Barrera</t>
   </si>
   <si>
@@ -376,51 +371,54 @@
     <t>High</t>
   </si>
   <si>
+    <t>Evaluado</t>
+  </si>
+  <si>
+    <t>Navegación pública</t>
+  </si>
+  <si>
+    <t>Los enlaces dirigen a la sección correspondiente.</t>
+  </si>
+  <si>
+    <t>El 100 % de enlaces principales funciona.</t>
+  </si>
+  <si>
+    <t>Prueba de navegación y capturas.</t>
+  </si>
+  <si>
+    <t>Mario Luzardo Fierro</t>
+  </si>
+  <si>
+    <t>Registro de usuarios</t>
+  </si>
+  <si>
+    <t>El visitante puede registrar una cuenta.</t>
+  </si>
+  <si>
+    <t>La cuenta se almacena cuando los datos son válidos.</t>
+  </si>
+  <si>
+    <t>Prueba funcional y registro en base de datos.</t>
+  </si>
+  <si>
+    <t>Highest</t>
+  </si>
+  <si>
+    <t>Validación de registro</t>
+  </si>
+  <si>
+    <t>El sistema rechaza datos incompletos o incorrectos.</t>
+  </si>
+  <si>
+    <t>Los campos obligatorios y formatos inválidos generan mensajes.</t>
+  </si>
+  <si>
+    <t>Pruebas positivas y negativas.</t>
+  </si>
+  <si>
     <t>Pendiente</t>
   </si>
   <si>
-    <t>Navegación pública</t>
-  </si>
-  <si>
-    <t>Los enlaces dirigen a la sección correspondiente.</t>
-  </si>
-  <si>
-    <t>El 100 % de enlaces principales funciona.</t>
-  </si>
-  <si>
-    <t>Prueba de navegación y capturas.</t>
-  </si>
-  <si>
-    <t>Mario Luzardo Fierro</t>
-  </si>
-  <si>
-    <t>Registro de usuarios</t>
-  </si>
-  <si>
-    <t>El visitante puede registrar una cuenta.</t>
-  </si>
-  <si>
-    <t>La cuenta se almacena cuando los datos son válidos.</t>
-  </si>
-  <si>
-    <t>Prueba funcional y registro en base de datos.</t>
-  </si>
-  <si>
-    <t>Highest</t>
-  </si>
-  <si>
-    <t>Validación de registro</t>
-  </si>
-  <si>
-    <t>El sistema rechaza datos incompletos o incorrectos.</t>
-  </si>
-  <si>
-    <t>Los campos obligatorios y formatos inválidos generan mensajes.</t>
-  </si>
-  <si>
-    <t>Pruebas positivas y negativas.</t>
-  </si>
-  <si>
     <t>Correo único</t>
   </si>
   <si>
@@ -1162,9 +1160,6 @@
     <t>10 MVP.pdf</t>
   </si>
   <si>
-    <t>Evaluado</t>
-  </si>
-  <si>
     <t>En proceso</t>
   </si>
   <si>
@@ -1181,13 +1176,316 @@
   </si>
   <si>
     <t>Ing. Victoria García Velásquez</t>
+  </si>
+  <si>
+    <t>1.1.0</t>
+  </si>
+  <si>
+    <t>19/09/2026</t>
+  </si>
+  <si>
+    <t>Incorporación de métricas con las columnas recomendadas por la docente.</t>
+  </si>
+  <si>
+    <t>Versión: 1.1.0</t>
+  </si>
+  <si>
+    <t>Actualización: 19/09/2026</t>
+  </si>
+  <si>
+    <t>MÉTRICAS DE CALIDAD DEL MVP</t>
+  </si>
+  <si>
+    <t>Estructura adaptada de la plantilla S06 Métricas de Calidad proporcionada para el Sprint 3</t>
+  </si>
+  <si>
+    <t>Las métricas permiten verificar el desempeño del proyecto y la calidad del MVP. Cada meta debe comprobarse con la fuente indicada y dentro del proceso correspondiente.</t>
+  </si>
+  <si>
+    <t>Nro</t>
+  </si>
+  <si>
+    <t>Qué queremos medir</t>
+  </si>
+  <si>
+    <t>Objetivo de Proyecto</t>
+  </si>
+  <si>
+    <t>Métrica</t>
+  </si>
+  <si>
+    <t>Meta</t>
+  </si>
+  <si>
+    <t>Fuente de datos</t>
+  </si>
+  <si>
+    <t>Proceso</t>
+  </si>
+  <si>
+    <t>Cumplimiento del cronograma del Sprint</t>
+  </si>
+  <si>
+    <t>Determinar si las actividades planificadas se completan dentro del periodo establecido.</t>
+  </si>
+  <si>
+    <t>SPI = avance ejecutado / avance planificado</t>
+  </si>
+  <si>
+    <t>≥ 0,95</t>
+  </si>
+  <si>
+    <t>Jira y Plan de Seguimiento del Sprint</t>
+  </si>
+  <si>
+    <t>Control del cronograma</t>
+  </si>
+  <si>
+    <t>Cumplimiento del alcance del MVP</t>
+  </si>
+  <si>
+    <t>Verificar que el desarrollo priorizado corresponda con el alcance aprobado del MVP.</t>
+  </si>
+  <si>
+    <t>Requisitos del MVP implementados y aceptados / requisitos planificados</t>
+  </si>
+  <si>
+    <t>≥ 95 % y ningún requisito crítico omitido</t>
+  </si>
+  <si>
+    <t>Documento MVP, Product Backlog y Jira</t>
+  </si>
+  <si>
+    <t>Gestión del alcance</t>
+  </si>
+  <si>
+    <t>Cumplimiento de requisitos funcionales</t>
+  </si>
+  <si>
+    <t>Comprobar que las funciones desarrolladas respondan a los requisitos aprobados.</t>
+  </si>
+  <si>
+    <t>Requisitos funcionales conformes / requisitos funcionales evaluados</t>
+  </si>
+  <si>
+    <t>≥ 95 %</t>
+  </si>
+  <si>
+    <t>Especificación de Requerimientos y resultados de pruebas</t>
+  </si>
+  <si>
+    <t>Control de calidad</t>
+  </si>
+  <si>
+    <t>Aprobación de pruebas funcionales</t>
+  </si>
+  <si>
+    <t>Medir la proporción de casos de prueba ejecutados satisfactoriamente.</t>
+  </si>
+  <si>
+    <t>Casos de prueba aprobados / casos de prueba ejecutados</t>
+  </si>
+  <si>
+    <t>≥ 95 % y 100 % de los casos Highest</t>
+  </si>
+  <si>
+    <t>Plan de pruebas, evidencias y registro de defectos</t>
+  </si>
+  <si>
+    <t>Aseguramiento de la calidad</t>
+  </si>
+  <si>
+    <t>Cierre de defectos y observaciones</t>
+  </si>
+  <si>
+    <t>Medir la atención de defectos y observaciones generados durante las revisiones.</t>
+  </si>
+  <si>
+    <t>Defectos cerrados y verificados / defectos registrados</t>
+  </si>
+  <si>
+    <t>≥ 90 % y 100 % de defectos críticos</t>
+  </si>
+  <si>
+    <t>Jira, registro de incidencias y evidencias de corrección</t>
+  </si>
+  <si>
+    <t>Gestión de la calidad</t>
+  </si>
+  <si>
+    <t>Cumplimiento de controles de seguridad</t>
+  </si>
+  <si>
+    <t>Verificar autenticación, autorización, protección de contraseñas y manejo seguro de datos.</t>
+  </si>
+  <si>
+    <t>Controles de seguridad conformes / controles evaluados</t>
+  </si>
+  <si>
+    <t>100 % de controles Highest y ≥ 95 % total</t>
+  </si>
+  <si>
+    <t>Matriz de calidad, pruebas de seguridad y revisión de código</t>
+  </si>
+  <si>
+    <t>Seguridad del software</t>
+  </si>
+  <si>
+    <t>Cumplimiento de accesibilidad</t>
+  </si>
+  <si>
+    <t>Verificar que las pantallas priorizadas sean comprensibles y operables por distintos usuarios.</t>
+  </si>
+  <si>
+    <t>Criterios de accesibilidad conformes / criterios evaluados</t>
+  </si>
+  <si>
+    <t>≥ 90 % y sin incumplimientos críticos</t>
+  </si>
+  <si>
+    <t>Lista de verificación WCAG, pruebas de teclado y capturas</t>
+  </si>
+  <si>
+    <t>Diseño y accesibilidad</t>
+  </si>
+  <si>
+    <t>Consistencia visual del producto</t>
+  </si>
+  <si>
+    <t>Comprobar la aplicación de colores, tipografía, encabezados y componentes definidos.</t>
+  </si>
+  <si>
+    <t>Pantallas conformes con lineamientos visuales / pantallas revisadas</t>
+  </si>
+  <si>
+    <t>Wireframes, CSS, lineamientos visuales y capturas</t>
+  </si>
+  <si>
+    <t>Diseño UI/UX</t>
+  </si>
+  <si>
+    <t>Rendimiento de páginas y servicios</t>
+  </si>
+  <si>
+    <t>Verificar que las funciones principales respondan en tiempos aceptables.</t>
+  </si>
+  <si>
+    <t>Tiempo promedio de carga de páginas y respuesta de servicios</t>
+  </si>
+  <si>
+    <t>Páginas ≤ 3 s; servicios principales ≤ 2 s en pruebas</t>
+  </si>
+  <si>
+    <t>Herramientas del navegador y registros de tiempos</t>
+  </si>
+  <si>
+    <t>Control del rendimiento</t>
+  </si>
+  <si>
+    <t>Trazabilidad de requisitos</t>
+  </si>
+  <si>
+    <t>Confirmar la relación entre requisitos, historias, pantallas, clases, código y pruebas.</t>
+  </si>
+  <si>
+    <t>Requisitos con trazabilidad completa / requisitos del MVP</t>
+  </si>
+  <si>
+    <t>100 %</t>
+  </si>
+  <si>
+    <t>Matriz de trazabilidad, Jira, modelos y repositorio Git</t>
+  </si>
+  <si>
+    <t>Gestión de requisitos</t>
+  </si>
+  <si>
+    <t>Cumplimiento documental</t>
+  </si>
+  <si>
+    <t>Medir el cumplimiento de estructura, versionamiento, coherencia y entregables académicos.</t>
+  </si>
+  <si>
+    <t>Documentos conformes / documentos revisados</t>
+  </si>
+  <si>
+    <t>≥ 97 %</t>
+  </si>
+  <si>
+    <t>Lista de revisión, Documento de Visión y repositorio documental</t>
+  </si>
+  <si>
+    <t>Gestión documental</t>
+  </si>
+  <si>
+    <t>Mantenibilidad del código</t>
+  </si>
+  <si>
+    <t>Verificar estructura, convenciones, documentación técnica y ausencia de duplicación relevante.</t>
+  </si>
+  <si>
+    <t>Criterios de mantenibilidad conformes / criterios evaluados</t>
+  </si>
+  <si>
+    <t>≥ 90 %</t>
+  </si>
+  <si>
+    <t>Revisión de código, README y repositorio Git</t>
+  </si>
+  <si>
+    <t>Desarrollo de software</t>
+  </si>
+  <si>
+    <t>Evidencias de actividades completadas</t>
+  </si>
+  <si>
+    <t>Comprobar que las tareas finalizadas cuenten con evidencia suficiente.</t>
+  </si>
+  <si>
+    <t>Tareas cerradas con evidencia / tareas cerradas</t>
+  </si>
+  <si>
+    <t>Jira, repositorio documental y Git</t>
+  </si>
+  <si>
+    <t>Seguimiento del proyecto</t>
+  </si>
+  <si>
+    <t>Gestión de riesgos y cambios</t>
+  </si>
+  <si>
+    <t>Verificar que los riesgos y cambios relevantes sean analizados, tratados y documentados.</t>
+  </si>
+  <si>
+    <t>Riesgos y cambios con tratamiento registrado / riesgos y cambios identificados</t>
+  </si>
+  <si>
+    <t>100 % de elementos altos o críticos y ≥ 95 % total</t>
+  </si>
+  <si>
+    <t>Matriz de riesgos y registro de gestión de cambios</t>
+  </si>
+  <si>
+    <t>Aceptación de entregables</t>
+  </si>
+  <si>
+    <t>Medir la aceptación de los resultados revisados por el Product Owner y la patrocinadora académica.</t>
+  </si>
+  <si>
+    <t>Entregables aceptados / entregables presentados</t>
+  </si>
+  <si>
+    <t>Actas, revisiones, Jira y registros de aprobación</t>
+  </si>
+  <si>
+    <t>Validación y aceptación</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -1262,8 +1560,14 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF212937"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1285,8 +1589,28 @@
         <fgColor rgb="FFC92351"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2A3966"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC92351"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -1597,11 +1921,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1699,6 +2038,21 @@
     <xf numFmtId="14" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1707,10 +2061,34 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1738,29 +2116,23 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1773,7 +2145,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
@@ -1784,7 +2156,7 @@
         <color rgb="FF7F6000"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -1795,7 +2167,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -1806,7 +2178,7 @@
         <color rgb="FF1B5E20"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
@@ -1817,7 +2189,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -1828,7 +2200,7 @@
         <color rgb="FF1B5E20"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
@@ -1838,7 +2210,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
@@ -1849,7 +2221,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -1860,7 +2232,7 @@
         <color rgb="FF7F6000"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -1870,7 +2242,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
@@ -1880,7 +2252,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFDCE6F1"/>
         </patternFill>
       </fill>
@@ -1891,7 +2263,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFCE4D6"/>
         </patternFill>
       </fill>
@@ -1902,7 +2274,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -1913,7 +2285,7 @@
         <color rgb="FF212937"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9D9D9"/>
         </patternFill>
       </fill>
@@ -1924,7 +2296,7 @@
         <color rgb="FF7F6000"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
@@ -1935,7 +2307,7 @@
         <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
@@ -1946,7 +2318,7 @@
         <color rgb="FF1B5E20"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
@@ -1981,10 +2353,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 4" descr="Student review [2955] for Universidad Espíritu Santo">
+        <xdr:cNvPr id="2" name="/xl/media/image1.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C9EC4C5B-7D34-B097-DE1B-299D560839A3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1992,34 +2364,16 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8696" t="18662" r="8925" b="19014"/>
-        <a:stretch/>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="142875" y="66675"/>
-          <a:ext cx="904875" cy="443865"/>
-        </a:xfrm>
+      <xdr:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
-            <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2044,10 +2398,10 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 4" descr="Student review [2955] for Universidad Espíritu Santo">
+        <xdr:cNvPr id="2" name="/xl/media/image1.jpeg">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F8728478-DA07-A5DB-B25B-0EAB65158349}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2055,34 +2409,16 @@
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
-      <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect l="8696" t="18662" r="8925" b="19014"/>
-        <a:stretch/>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
       </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="114300" y="76200"/>
-          <a:ext cx="906780" cy="445770"/>
-        </a:xfrm>
+      <xdr:spPr>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{53640926-AAD7-44D8-BBD7-CCE9431645EC}">
-            <a14:shadowObscured xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main"/>
-          </a:ext>
-        </a:extLst>
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
@@ -2327,35 +2663,35 @@
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="39" t="s">
+      <c r="B1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
-      <c r="K1" s="40"/>
-      <c r="L1" s="40"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
       <c r="A2" s="12"/>
-      <c r="B2" s="41" t="s">
+      <c r="B2" s="46" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="42"/>
-      <c r="J2" s="42"/>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">
       <c r="A3" s="13"/>
@@ -2880,6 +3216,23 @@
         <v>59</v>
       </c>
     </row>
+    <row r="26" spans="1:5" ht="34.049999999999997" customHeight="1">
+      <c r="A26" s="42" t="s">
+        <v>380</v>
+      </c>
+      <c r="B26" s="42" t="s">
+        <v>381</v>
+      </c>
+      <c r="C26" s="42" t="s">
+        <v>382</v>
+      </c>
+      <c r="D26" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="42" t="s">
+        <v>59</v>
+      </c>
+    </row>
     <row r="27" spans="1:5">
       <c r="A27" s="2" t="s">
         <v>60</v>
@@ -2917,7 +3270,7 @@
         <v>68</v>
       </c>
       <c r="B31" s="34" t="s">
-        <v>56</v>
+        <v>380</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -2941,7 +3294,7 @@
         <v>71</v>
       </c>
       <c r="B34" s="37">
-        <v>46279</v>
+        <v>46284</v>
       </c>
     </row>
     <row r="35" spans="1:2">
@@ -3012,6 +3365,13 @@
       </dataBar>
     </cfRule>
     <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFC92351"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="7">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3075,98 +3435,98 @@
     <row r="1" spans="1:17" ht="25.05" customHeight="1">
       <c r="A1" s="12"/>
       <c r="B1" s="12"/>
-      <c r="C1" s="58" t="s">
+      <c r="C1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
-      <c r="P1" s="42"/>
-      <c r="Q1" s="42"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
     </row>
     <row r="2" spans="1:17" ht="25.05" customHeight="1">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
-      <c r="C2" s="41" t="s">
+      <c r="C2" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
-      <c r="P2" s="44"/>
-      <c r="Q2" s="44"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
+      <c r="P2" s="49"/>
+      <c r="Q2" s="49"/>
     </row>
     <row r="3" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A3" s="59" t="s">
+      <c r="A3" s="50" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="D3" s="60"/>
-      <c r="E3" s="60" t="s">
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51" t="s">
+        <v>383</v>
+      </c>
+      <c r="F3" s="51"/>
+      <c r="G3" s="51"/>
+      <c r="H3" s="51"/>
+      <c r="I3" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="F3" s="60"/>
-      <c r="G3" s="60"/>
-      <c r="H3" s="60"/>
-      <c r="I3" s="60" t="s">
+      <c r="J3" s="51"/>
+      <c r="K3" s="51"/>
+      <c r="L3" s="51" t="s">
+        <v>384</v>
+      </c>
+      <c r="M3" s="51"/>
+      <c r="N3" s="51"/>
+      <c r="O3" s="51"/>
+      <c r="P3" s="51"/>
+      <c r="Q3" s="52"/>
+    </row>
+    <row r="4" spans="1:17" ht="22.05" customHeight="1">
+      <c r="A4" s="53" t="s">
         <v>84</v>
       </c>
-      <c r="J3" s="60"/>
-      <c r="K3" s="60"/>
-      <c r="L3" s="60"/>
-      <c r="M3" s="60" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="N3" s="60"/>
-      <c r="O3" s="60"/>
-      <c r="P3" s="60"/>
-      <c r="Q3" s="61"/>
-    </row>
-    <row r="4" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A4" s="54" t="s">
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54" t="s">
         <v>86</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55" t="s">
+      <c r="J4" s="54"/>
+      <c r="K4" s="54"/>
+      <c r="L4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
-      <c r="I4" s="55" t="s">
-        <v>88</v>
-      </c>
-      <c r="J4" s="55"/>
-      <c r="K4" s="55"/>
-      <c r="L4" s="55"/>
-      <c r="M4" s="55" t="s">
-        <v>89</v>
-      </c>
-      <c r="N4" s="55"/>
-      <c r="O4" s="55"/>
-      <c r="P4" s="55"/>
-      <c r="Q4" s="56"/>
+      <c r="N4" s="54"/>
+      <c r="O4" s="54"/>
+      <c r="P4" s="54"/>
+      <c r="Q4" s="55"/>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="13"/>
@@ -3188,185 +3548,185 @@
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="24" customHeight="1">
-      <c r="A6" s="57" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="44"/>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
-      <c r="H6" s="44"/>
-      <c r="I6" s="44"/>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44"/>
-      <c r="L6" s="44"/>
-      <c r="M6" s="44"/>
-      <c r="N6" s="44"/>
-      <c r="O6" s="44"/>
-      <c r="P6" s="44"/>
-      <c r="Q6" s="44"/>
+      <c r="A6" s="56" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="49"/>
+      <c r="C6" s="49"/>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="F6" s="49"/>
+      <c r="G6" s="49"/>
+      <c r="H6" s="49"/>
+      <c r="I6" s="49"/>
+      <c r="J6" s="49"/>
+      <c r="K6" s="49"/>
+      <c r="L6" s="49"/>
+      <c r="M6" s="49"/>
+      <c r="N6" s="49"/>
+      <c r="O6" s="49"/>
+      <c r="P6" s="49"/>
+      <c r="Q6" s="49"/>
     </row>
     <row r="7" spans="1:17" ht="24" customHeight="1">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="45"/>
+      <c r="B7" s="58"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="45"/>
+      <c r="E7" s="58"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="45"/>
+      <c r="H7" s="58"/>
       <c r="I7" s="14"/>
-      <c r="J7" s="45" t="s">
+      <c r="J7" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="45"/>
+      <c r="K7" s="58"/>
       <c r="L7" s="14"/>
-      <c r="M7" s="45" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" s="45"/>
+      <c r="M7" s="58" t="s">
+        <v>89</v>
+      </c>
+      <c r="N7" s="58"/>
       <c r="O7" s="14"/>
-      <c r="P7" s="45" t="s">
+      <c r="P7" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="Q7" s="45"/>
+      <c r="Q7" s="58"/>
     </row>
     <row r="8" spans="1:17" ht="24" customHeight="1">
-      <c r="A8" s="46">
+      <c r="A8" s="59">
         <f>COUNTA(A13:A76)</f>
         <v>64</v>
       </c>
-      <c r="B8" s="47"/>
+      <c r="B8" s="60"/>
       <c r="C8" s="15"/>
-      <c r="D8" s="47">
+      <c r="D8" s="60">
         <f>COUNTIF(I13:I76,"Cumple")+COUNTIF(I13:I76,"Cumple parcialmente")+COUNTIF(I13:I76,"No cumple")+COUNTIF(I13:I76,"No aplica")</f>
         <v>2</v>
       </c>
-      <c r="E8" s="47"/>
+      <c r="E8" s="60"/>
       <c r="F8" s="15"/>
-      <c r="G8" s="50">
+      <c r="G8" s="63">
         <f>IFERROR(D8/A8,0)</f>
         <v>3.125E-2</v>
       </c>
-      <c r="H8" s="50"/>
+      <c r="H8" s="63"/>
       <c r="I8" s="15"/>
-      <c r="J8" s="50">
+      <c r="J8" s="63">
         <f>IFERROR(SUM(J13:J76)/(COUNT(J13:J76)*2),0)</f>
         <v>1</v>
       </c>
-      <c r="K8" s="50"/>
+      <c r="K8" s="63"/>
       <c r="L8" s="15"/>
-      <c r="M8" s="50">
+      <c r="M8" s="63">
         <f>IFERROR(COUNTIF(I13:I76,"Cumple")/COUNT(J13:J76),0)</f>
         <v>1</v>
       </c>
-      <c r="N8" s="50"/>
+      <c r="N8" s="63"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="47" t="str">
+      <c r="P8" s="60" t="str">
         <f>IF(G8&lt;1,"PENDIENTE DE EVALUACIÓN",IF(COUNTIFS(G13:G76,"Highest",I13:I76,"No cumple")&gt;0,"NO APROBADO",IF(J8&gt;=0.9,"APROBADO","REQUIERE MEJORAS")))</f>
         <v>PENDIENTE DE EVALUACIÓN</v>
       </c>
-      <c r="Q8" s="52"/>
+      <c r="Q8" s="65"/>
     </row>
     <row r="9" spans="1:17" ht="24" customHeight="1">
-      <c r="A9" s="48"/>
-      <c r="B9" s="49"/>
+      <c r="A9" s="61"/>
+      <c r="B9" s="62"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
       <c r="F9" s="16"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
+      <c r="G9" s="64"/>
+      <c r="H9" s="64"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
+      <c r="J9" s="64"/>
+      <c r="K9" s="64"/>
       <c r="L9" s="16"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="51"/>
+      <c r="M9" s="64"/>
+      <c r="N9" s="64"/>
       <c r="O9" s="16"/>
-      <c r="P9" s="49"/>
-      <c r="Q9" s="53"/>
+      <c r="P9" s="62"/>
+      <c r="Q9" s="66"/>
     </row>
     <row r="10" spans="1:17" ht="24" customHeight="1">
-      <c r="A10" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
-      <c r="P10" s="44"/>
-      <c r="Q10" s="44"/>
+      <c r="A10" s="57" t="s">
+        <v>90</v>
+      </c>
+      <c r="B10" s="49"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="49"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="49"/>
+      <c r="I10" s="49"/>
+      <c r="J10" s="49"/>
+      <c r="K10" s="49"/>
+      <c r="L10" s="49"/>
+      <c r="M10" s="49"/>
+      <c r="N10" s="49"/>
+      <c r="O10" s="49"/>
+      <c r="P10" s="49"/>
+      <c r="Q10" s="49"/>
     </row>
     <row r="12" spans="1:17" ht="42" customHeight="1">
       <c r="A12" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="E12" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="D12" s="18" t="s">
+      <c r="F12" s="18" t="s">
         <v>95</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="G12" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="F12" s="18" t="s">
+      <c r="H12" s="18" t="s">
         <v>97</v>
-      </c>
-      <c r="G12" s="18" t="s">
-        <v>98</v>
-      </c>
-      <c r="H12" s="18" t="s">
-        <v>99</v>
       </c>
       <c r="I12" s="18" t="s">
         <v>3</v>
       </c>
       <c r="J12" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>99</v>
+      </c>
+      <c r="L12" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="M12" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="L12" s="18" t="s">
+      <c r="N12" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="M12" s="18" t="s">
+      <c r="O12" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="N12" s="18" t="s">
+      <c r="P12" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="O12" s="18" t="s">
+      <c r="Q12" s="19" t="s">
         <v>105</v>
-      </c>
-      <c r="P12" s="18" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q12" s="19" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="58.05" customHeight="1">
@@ -3374,25 +3734,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="E13" s="20" t="s">
         <v>109</v>
-      </c>
-      <c r="D13" s="20" t="s">
-        <v>110</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>111</v>
       </c>
       <c r="F13" s="20" t="s">
         <v>38</v>
       </c>
       <c r="G13" s="20" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H13" s="20" t="s">
-        <v>375</v>
+        <v>111</v>
       </c>
       <c r="I13" s="20" t="s">
         <v>7</v>
@@ -3414,25 +3774,25 @@
         <v>12</v>
       </c>
       <c r="B14" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="E14" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="F14" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="E14" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="21" t="s">
-        <v>118</v>
-      </c>
       <c r="G14" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H14" s="21" t="s">
-        <v>375</v>
+        <v>111</v>
       </c>
       <c r="I14" s="21"/>
       <c r="J14" s="21" t="str">
@@ -3452,25 +3812,25 @@
         <v>12</v>
       </c>
       <c r="B15" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="E15" s="21" t="s">
         <v>120</v>
-      </c>
-      <c r="D15" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="E15" s="21" t="s">
-        <v>122</v>
       </c>
       <c r="F15" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G15" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H15" s="21" t="s">
-        <v>375</v>
+        <v>111</v>
       </c>
       <c r="I15" s="21" t="s">
         <v>7</v>
@@ -3492,25 +3852,25 @@
         <v>12</v>
       </c>
       <c r="B16" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="E16" s="21" t="s">
         <v>125</v>
-      </c>
-      <c r="D16" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="E16" s="21" t="s">
-        <v>127</v>
       </c>
       <c r="F16" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G16" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I16" s="21"/>
       <c r="J16" s="21" t="str">
@@ -3530,25 +3890,25 @@
         <v>12</v>
       </c>
       <c r="B17" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="D17" s="21" t="s">
+      <c r="E17" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="F17" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="F17" s="21" t="s">
-        <v>132</v>
-      </c>
       <c r="G17" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H17" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I17" s="21"/>
       <c r="J17" s="21" t="str">
@@ -3568,25 +3928,25 @@
         <v>12</v>
       </c>
       <c r="B18" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="D18" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="E18" s="21" t="s">
         <v>135</v>
-      </c>
-      <c r="E18" s="21" t="s">
-        <v>136</v>
       </c>
       <c r="F18" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G18" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H18" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I18" s="21"/>
       <c r="J18" s="21" t="str">
@@ -3606,25 +3966,25 @@
         <v>12</v>
       </c>
       <c r="B19" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="C19" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="D19" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="E19" s="21" t="s">
         <v>139</v>
-      </c>
-      <c r="E19" s="21" t="s">
-        <v>140</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G19" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H19" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I19" s="21"/>
       <c r="J19" s="21" t="str">
@@ -3644,25 +4004,25 @@
         <v>12</v>
       </c>
       <c r="B20" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C20" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="D20" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="D20" s="21" t="s">
+      <c r="E20" s="21" t="s">
         <v>143</v>
-      </c>
-      <c r="E20" s="21" t="s">
-        <v>144</v>
       </c>
       <c r="F20" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G20" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H20" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I20" s="21"/>
       <c r="J20" s="21" t="str">
@@ -3682,25 +4042,25 @@
         <v>12</v>
       </c>
       <c r="B21" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="D21" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="D21" s="21" t="s">
+      <c r="E21" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="E21" s="21" t="s">
-        <v>148</v>
-      </c>
       <c r="F21" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G21" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H21" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I21" s="21"/>
       <c r="J21" s="21" t="str">
@@ -3720,25 +4080,25 @@
         <v>12</v>
       </c>
       <c r="B22" s="21" t="s">
+        <v>148</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="D22" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="E22" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="E22" s="21" t="s">
-        <v>152</v>
-      </c>
       <c r="F22" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G22" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H22" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I22" s="21"/>
       <c r="J22" s="21" t="str">
@@ -3758,25 +4118,25 @@
         <v>12</v>
       </c>
       <c r="B23" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="21" t="s">
+      <c r="D23" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="D23" s="21" t="s">
+      <c r="E23" s="21" t="s">
         <v>155</v>
-      </c>
-      <c r="E23" s="21" t="s">
-        <v>156</v>
       </c>
       <c r="F23" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G23" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I23" s="21"/>
       <c r="J23" s="21" t="str">
@@ -3796,25 +4156,25 @@
         <v>12</v>
       </c>
       <c r="B24" s="21" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="D24" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="D24" s="21" t="s">
+      <c r="E24" s="21" t="s">
         <v>159</v>
-      </c>
-      <c r="E24" s="21" t="s">
-        <v>160</v>
       </c>
       <c r="F24" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G24" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H24" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I24" s="21"/>
       <c r="J24" s="21" t="str">
@@ -3834,25 +4194,25 @@
         <v>14</v>
       </c>
       <c r="B25" s="21" t="s">
+        <v>160</v>
+      </c>
+      <c r="C25" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="D25" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="D25" s="21" t="s">
+      <c r="E25" s="21" t="s">
         <v>163</v>
-      </c>
-      <c r="E25" s="21" t="s">
-        <v>164</v>
       </c>
       <c r="F25" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G25" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I25" s="21"/>
       <c r="J25" s="21" t="str">
@@ -3872,25 +4232,25 @@
         <v>14</v>
       </c>
       <c r="B26" s="21" t="s">
+        <v>164</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="D26" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="E26" s="21" t="s">
         <v>167</v>
-      </c>
-      <c r="E26" s="21" t="s">
-        <v>168</v>
       </c>
       <c r="F26" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G26" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H26" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I26" s="21"/>
       <c r="J26" s="21" t="str">
@@ -3910,25 +4270,25 @@
         <v>14</v>
       </c>
       <c r="B27" s="21" t="s">
+        <v>168</v>
+      </c>
+      <c r="C27" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="C27" s="21" t="s">
+      <c r="D27" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="D27" s="21" t="s">
+      <c r="E27" s="21" t="s">
         <v>171</v>
-      </c>
-      <c r="E27" s="21" t="s">
-        <v>172</v>
       </c>
       <c r="F27" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H27" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I27" s="21"/>
       <c r="J27" s="21" t="str">
@@ -3948,25 +4308,25 @@
         <v>14</v>
       </c>
       <c r="B28" s="21" t="s">
+        <v>172</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="D28" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="D28" s="21" t="s">
+      <c r="E28" s="21" t="s">
         <v>175</v>
-      </c>
-      <c r="E28" s="21" t="s">
-        <v>176</v>
       </c>
       <c r="F28" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G28" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H28" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I28" s="21"/>
       <c r="J28" s="21" t="str">
@@ -3986,25 +4346,25 @@
         <v>14</v>
       </c>
       <c r="B29" s="21" t="s">
+        <v>176</v>
+      </c>
+      <c r="C29" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="C29" s="21" t="s">
+      <c r="D29" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="D29" s="21" t="s">
+      <c r="E29" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="E29" s="21" t="s">
-        <v>180</v>
-      </c>
       <c r="F29" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G29" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I29" s="21"/>
       <c r="J29" s="21" t="str">
@@ -4024,25 +4384,25 @@
         <v>14</v>
       </c>
       <c r="B30" s="21" t="s">
+        <v>180</v>
+      </c>
+      <c r="C30" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="D30" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="E30" s="21" t="s">
         <v>183</v>
-      </c>
-      <c r="E30" s="21" t="s">
-        <v>184</v>
       </c>
       <c r="F30" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G30" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H30" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I30" s="21"/>
       <c r="J30" s="21" t="str">
@@ -4062,25 +4422,25 @@
         <v>14</v>
       </c>
       <c r="B31" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="C31" s="21" t="s">
         <v>185</v>
       </c>
-      <c r="C31" s="21" t="s">
+      <c r="D31" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="D31" s="21" t="s">
+      <c r="E31" s="21" t="s">
         <v>187</v>
-      </c>
-      <c r="E31" s="21" t="s">
-        <v>188</v>
       </c>
       <c r="F31" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G31" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H31" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I31" s="21"/>
       <c r="J31" s="21" t="str">
@@ -4100,25 +4460,25 @@
         <v>14</v>
       </c>
       <c r="B32" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="C32" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="D32" s="21" t="s">
         <v>190</v>
       </c>
-      <c r="D32" s="21" t="s">
+      <c r="E32" s="21" t="s">
         <v>191</v>
       </c>
-      <c r="E32" s="21" t="s">
+      <c r="F32" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="G32" s="21" t="s">
         <v>192</v>
       </c>
-      <c r="F32" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="G32" s="21" t="s">
-        <v>193</v>
-      </c>
       <c r="H32" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I32" s="21"/>
       <c r="J32" s="21" t="str">
@@ -4138,25 +4498,25 @@
         <v>14</v>
       </c>
       <c r="B33" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="D33" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="D33" s="21" t="s">
+      <c r="E33" s="21" t="s">
         <v>196</v>
-      </c>
-      <c r="E33" s="21" t="s">
-        <v>197</v>
       </c>
       <c r="F33" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G33" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H33" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I33" s="21"/>
       <c r="J33" s="21" t="str">
@@ -4176,25 +4536,25 @@
         <v>16</v>
       </c>
       <c r="B34" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="C34" s="21" t="s">
         <v>198</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="D34" s="21" t="s">
         <v>199</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="E34" s="21" t="s">
         <v>200</v>
-      </c>
-      <c r="E34" s="21" t="s">
-        <v>201</v>
       </c>
       <c r="F34" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G34" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H34" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I34" s="21"/>
       <c r="J34" s="21" t="str">
@@ -4214,25 +4574,25 @@
         <v>16</v>
       </c>
       <c r="B35" s="21" t="s">
+        <v>201</v>
+      </c>
+      <c r="C35" s="21" t="s">
         <v>202</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="D35" s="21" t="s">
         <v>203</v>
       </c>
-      <c r="D35" s="21" t="s">
+      <c r="E35" s="21" t="s">
         <v>204</v>
-      </c>
-      <c r="E35" s="21" t="s">
-        <v>205</v>
       </c>
       <c r="F35" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G35" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H35" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I35" s="21"/>
       <c r="J35" s="21" t="str">
@@ -4252,25 +4612,25 @@
         <v>16</v>
       </c>
       <c r="B36" s="21" t="s">
+        <v>205</v>
+      </c>
+      <c r="C36" s="21" t="s">
         <v>206</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="D36" s="21" t="s">
         <v>207</v>
       </c>
-      <c r="D36" s="21" t="s">
+      <c r="E36" s="21" t="s">
         <v>208</v>
       </c>
-      <c r="E36" s="21" t="s">
-        <v>209</v>
-      </c>
       <c r="F36" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G36" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H36" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I36" s="21"/>
       <c r="J36" s="21" t="str">
@@ -4290,25 +4650,25 @@
         <v>16</v>
       </c>
       <c r="B37" s="21" t="s">
+        <v>209</v>
+      </c>
+      <c r="C37" s="21" t="s">
         <v>210</v>
       </c>
-      <c r="C37" s="21" t="s">
+      <c r="D37" s="21" t="s">
         <v>211</v>
       </c>
-      <c r="D37" s="21" t="s">
+      <c r="E37" s="21" t="s">
         <v>212</v>
       </c>
-      <c r="E37" s="21" t="s">
-        <v>213</v>
-      </c>
       <c r="F37" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G37" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H37" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I37" s="21"/>
       <c r="J37" s="21" t="str">
@@ -4328,25 +4688,25 @@
         <v>16</v>
       </c>
       <c r="B38" s="21" t="s">
+        <v>213</v>
+      </c>
+      <c r="C38" s="21" t="s">
         <v>214</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="D38" s="21" t="s">
         <v>215</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="E38" s="21" t="s">
         <v>216</v>
-      </c>
-      <c r="E38" s="21" t="s">
-        <v>217</v>
       </c>
       <c r="F38" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G38" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H38" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I38" s="21"/>
       <c r="J38" s="21" t="str">
@@ -4366,25 +4726,25 @@
         <v>16</v>
       </c>
       <c r="B39" s="21" t="s">
+        <v>217</v>
+      </c>
+      <c r="C39" s="21" t="s">
         <v>218</v>
       </c>
-      <c r="C39" s="21" t="s">
+      <c r="D39" s="21" t="s">
         <v>219</v>
       </c>
-      <c r="D39" s="21" t="s">
+      <c r="E39" s="21" t="s">
         <v>220</v>
-      </c>
-      <c r="E39" s="21" t="s">
-        <v>221</v>
       </c>
       <c r="F39" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G39" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H39" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I39" s="21"/>
       <c r="J39" s="21" t="str">
@@ -4404,25 +4764,25 @@
         <v>16</v>
       </c>
       <c r="B40" s="21" t="s">
+        <v>221</v>
+      </c>
+      <c r="C40" s="21" t="s">
         <v>222</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="D40" s="21" t="s">
         <v>223</v>
       </c>
-      <c r="D40" s="21" t="s">
+      <c r="E40" s="21" t="s">
         <v>224</v>
       </c>
-      <c r="E40" s="21" t="s">
-        <v>225</v>
-      </c>
       <c r="F40" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G40" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H40" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I40" s="21"/>
       <c r="J40" s="21" t="str">
@@ -4442,25 +4802,25 @@
         <v>16</v>
       </c>
       <c r="B41" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="C41" s="21" t="s">
         <v>226</v>
       </c>
-      <c r="C41" s="21" t="s">
+      <c r="D41" s="21" t="s">
         <v>227</v>
       </c>
-      <c r="D41" s="21" t="s">
+      <c r="E41" s="21" t="s">
         <v>228</v>
       </c>
-      <c r="E41" s="21" t="s">
-        <v>229</v>
-      </c>
       <c r="F41" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G41" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H41" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I41" s="21"/>
       <c r="J41" s="21" t="str">
@@ -4480,25 +4840,25 @@
         <v>16</v>
       </c>
       <c r="B42" s="21" t="s">
+        <v>229</v>
+      </c>
+      <c r="C42" s="21" t="s">
         <v>230</v>
       </c>
-      <c r="C42" s="21" t="s">
+      <c r="D42" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="E42" s="21" t="s">
         <v>232</v>
       </c>
-      <c r="E42" s="21" t="s">
-        <v>233</v>
-      </c>
       <c r="F42" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G42" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H42" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I42" s="21"/>
       <c r="J42" s="21" t="str">
@@ -4518,25 +4878,25 @@
         <v>16</v>
       </c>
       <c r="B43" s="21" t="s">
+        <v>233</v>
+      </c>
+      <c r="C43" s="21" t="s">
         <v>234</v>
       </c>
-      <c r="C43" s="21" t="s">
+      <c r="D43" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="D43" s="21" t="s">
+      <c r="E43" s="21" t="s">
         <v>236</v>
-      </c>
-      <c r="E43" s="21" t="s">
-        <v>237</v>
       </c>
       <c r="F43" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G43" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H43" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I43" s="21"/>
       <c r="J43" s="21" t="str">
@@ -4556,25 +4916,25 @@
         <v>16</v>
       </c>
       <c r="B44" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="C44" s="21" t="s">
         <v>238</v>
       </c>
-      <c r="C44" s="21" t="s">
+      <c r="D44" s="21" t="s">
         <v>239</v>
       </c>
-      <c r="D44" s="21" t="s">
+      <c r="E44" s="21" t="s">
         <v>240</v>
-      </c>
-      <c r="E44" s="21" t="s">
-        <v>241</v>
       </c>
       <c r="F44" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G44" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H44" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I44" s="21"/>
       <c r="J44" s="21" t="str">
@@ -4594,25 +4954,25 @@
         <v>18</v>
       </c>
       <c r="B45" s="21" t="s">
+        <v>241</v>
+      </c>
+      <c r="C45" s="21" t="s">
         <v>242</v>
       </c>
-      <c r="C45" s="21" t="s">
+      <c r="D45" s="21" t="s">
         <v>243</v>
       </c>
-      <c r="D45" s="21" t="s">
+      <c r="E45" s="21" t="s">
         <v>244</v>
       </c>
-      <c r="E45" s="21" t="s">
-        <v>245</v>
-      </c>
       <c r="F45" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G45" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H45" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I45" s="21"/>
       <c r="J45" s="21" t="str">
@@ -4632,25 +4992,25 @@
         <v>18</v>
       </c>
       <c r="B46" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="C46" s="21" t="s">
         <v>246</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="D46" s="21" t="s">
         <v>247</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="E46" s="21" t="s">
         <v>248</v>
       </c>
-      <c r="E46" s="21" t="s">
-        <v>249</v>
-      </c>
       <c r="F46" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G46" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H46" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I46" s="21"/>
       <c r="J46" s="21" t="str">
@@ -4670,25 +5030,25 @@
         <v>18</v>
       </c>
       <c r="B47" s="21" t="s">
+        <v>249</v>
+      </c>
+      <c r="C47" s="21" t="s">
         <v>250</v>
       </c>
-      <c r="C47" s="21" t="s">
+      <c r="D47" s="21" t="s">
         <v>251</v>
       </c>
-      <c r="D47" s="21" t="s">
+      <c r="E47" s="21" t="s">
         <v>252</v>
       </c>
-      <c r="E47" s="21" t="s">
-        <v>253</v>
-      </c>
       <c r="F47" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G47" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H47" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I47" s="21"/>
       <c r="J47" s="21" t="str">
@@ -4708,25 +5068,25 @@
         <v>18</v>
       </c>
       <c r="B48" s="21" t="s">
+        <v>253</v>
+      </c>
+      <c r="C48" s="21" t="s">
         <v>254</v>
       </c>
-      <c r="C48" s="21" t="s">
+      <c r="D48" s="21" t="s">
         <v>255</v>
       </c>
-      <c r="D48" s="21" t="s">
+      <c r="E48" s="21" t="s">
         <v>256</v>
       </c>
-      <c r="E48" s="21" t="s">
-        <v>257</v>
-      </c>
       <c r="F48" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G48" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H48" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I48" s="21"/>
       <c r="J48" s="21" t="str">
@@ -4746,25 +5106,25 @@
         <v>18</v>
       </c>
       <c r="B49" s="21" t="s">
+        <v>257</v>
+      </c>
+      <c r="C49" s="21" t="s">
         <v>258</v>
       </c>
-      <c r="C49" s="21" t="s">
+      <c r="D49" s="21" t="s">
         <v>259</v>
       </c>
-      <c r="D49" s="21" t="s">
+      <c r="E49" s="21" t="s">
         <v>260</v>
-      </c>
-      <c r="E49" s="21" t="s">
-        <v>261</v>
       </c>
       <c r="F49" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G49" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H49" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I49" s="21"/>
       <c r="J49" s="21" t="str">
@@ -4784,25 +5144,25 @@
         <v>18</v>
       </c>
       <c r="B50" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="C50" s="21" t="s">
         <v>262</v>
       </c>
-      <c r="C50" s="21" t="s">
+      <c r="D50" s="21" t="s">
         <v>263</v>
       </c>
-      <c r="D50" s="21" t="s">
+      <c r="E50" s="21" t="s">
         <v>264</v>
       </c>
-      <c r="E50" s="21" t="s">
-        <v>265</v>
-      </c>
       <c r="F50" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G50" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H50" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I50" s="21"/>
       <c r="J50" s="21" t="str">
@@ -4822,25 +5182,25 @@
         <v>18</v>
       </c>
       <c r="B51" s="21" t="s">
+        <v>265</v>
+      </c>
+      <c r="C51" s="21" t="s">
         <v>266</v>
       </c>
-      <c r="C51" s="21" t="s">
+      <c r="D51" s="21" t="s">
         <v>267</v>
       </c>
-      <c r="D51" s="21" t="s">
+      <c r="E51" s="21" t="s">
         <v>268</v>
       </c>
-      <c r="E51" s="21" t="s">
-        <v>269</v>
-      </c>
       <c r="F51" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G51" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H51" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I51" s="21"/>
       <c r="J51" s="21" t="str">
@@ -4860,25 +5220,25 @@
         <v>18</v>
       </c>
       <c r="B52" s="21" t="s">
+        <v>269</v>
+      </c>
+      <c r="C52" s="21" t="s">
         <v>270</v>
       </c>
-      <c r="C52" s="21" t="s">
+      <c r="D52" s="21" t="s">
         <v>271</v>
       </c>
-      <c r="D52" s="21" t="s">
+      <c r="E52" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="E52" s="21" t="s">
-        <v>273</v>
-      </c>
       <c r="F52" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G52" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H52" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I52" s="21"/>
       <c r="J52" s="21" t="str">
@@ -4898,25 +5258,25 @@
         <v>18</v>
       </c>
       <c r="B53" s="21" t="s">
+        <v>273</v>
+      </c>
+      <c r="C53" s="21" t="s">
         <v>274</v>
       </c>
-      <c r="C53" s="21" t="s">
+      <c r="D53" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="D53" s="21" t="s">
-        <v>276</v>
-      </c>
       <c r="E53" s="21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F53" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G53" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H53" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I53" s="21"/>
       <c r="J53" s="21" t="str">
@@ -4936,25 +5296,25 @@
         <v>18</v>
       </c>
       <c r="B54" s="21" t="s">
+        <v>276</v>
+      </c>
+      <c r="C54" s="21" t="s">
         <v>277</v>
       </c>
-      <c r="C54" s="21" t="s">
+      <c r="D54" s="21" t="s">
         <v>278</v>
       </c>
-      <c r="D54" s="21" t="s">
+      <c r="E54" s="21" t="s">
         <v>279</v>
-      </c>
-      <c r="E54" s="21" t="s">
-        <v>280</v>
       </c>
       <c r="F54" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G54" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H54" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I54" s="21"/>
       <c r="J54" s="21" t="str">
@@ -4974,25 +5334,25 @@
         <v>20</v>
       </c>
       <c r="B55" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="C55" s="21" t="s">
         <v>281</v>
       </c>
-      <c r="C55" s="21" t="s">
+      <c r="D55" s="21" t="s">
         <v>282</v>
       </c>
-      <c r="D55" s="21" t="s">
+      <c r="E55" s="21" t="s">
         <v>283</v>
-      </c>
-      <c r="E55" s="21" t="s">
-        <v>284</v>
       </c>
       <c r="F55" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G55" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H55" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I55" s="21"/>
       <c r="J55" s="21" t="str">
@@ -5012,25 +5372,25 @@
         <v>20</v>
       </c>
       <c r="B56" s="21" t="s">
+        <v>284</v>
+      </c>
+      <c r="C56" s="21" t="s">
         <v>285</v>
       </c>
-      <c r="C56" s="21" t="s">
+      <c r="D56" s="21" t="s">
         <v>286</v>
       </c>
-      <c r="D56" s="21" t="s">
+      <c r="E56" s="21" t="s">
         <v>287</v>
       </c>
-      <c r="E56" s="21" t="s">
-        <v>288</v>
-      </c>
       <c r="F56" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G56" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H56" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I56" s="21"/>
       <c r="J56" s="21" t="str">
@@ -5050,25 +5410,25 @@
         <v>22</v>
       </c>
       <c r="B57" s="21" t="s">
+        <v>288</v>
+      </c>
+      <c r="C57" s="21" t="s">
         <v>289</v>
       </c>
-      <c r="C57" s="21" t="s">
+      <c r="D57" s="21" t="s">
         <v>290</v>
       </c>
-      <c r="D57" s="21" t="s">
+      <c r="E57" s="21" t="s">
         <v>291</v>
-      </c>
-      <c r="E57" s="21" t="s">
-        <v>292</v>
       </c>
       <c r="F57" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G57" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H57" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I57" s="21"/>
       <c r="J57" s="21" t="str">
@@ -5088,25 +5448,25 @@
         <v>22</v>
       </c>
       <c r="B58" s="21" t="s">
+        <v>292</v>
+      </c>
+      <c r="C58" s="21" t="s">
         <v>293</v>
       </c>
-      <c r="C58" s="21" t="s">
+      <c r="D58" s="21" t="s">
         <v>294</v>
       </c>
-      <c r="D58" s="21" t="s">
+      <c r="E58" s="21" t="s">
         <v>295</v>
       </c>
-      <c r="E58" s="21" t="s">
-        <v>296</v>
-      </c>
       <c r="F58" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G58" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H58" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I58" s="21"/>
       <c r="J58" s="21" t="str">
@@ -5126,25 +5486,25 @@
         <v>24</v>
       </c>
       <c r="B59" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="C59" s="21" t="s">
         <v>297</v>
       </c>
-      <c r="C59" s="21" t="s">
+      <c r="D59" s="21" t="s">
         <v>298</v>
       </c>
-      <c r="D59" s="21" t="s">
+      <c r="E59" s="21" t="s">
         <v>299</v>
       </c>
-      <c r="E59" s="21" t="s">
-        <v>300</v>
-      </c>
       <c r="F59" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G59" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H59" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I59" s="21"/>
       <c r="J59" s="21" t="str">
@@ -5164,25 +5524,25 @@
         <v>24</v>
       </c>
       <c r="B60" s="21" t="s">
+        <v>300</v>
+      </c>
+      <c r="C60" s="21" t="s">
         <v>301</v>
       </c>
-      <c r="C60" s="21" t="s">
+      <c r="D60" s="21" t="s">
         <v>302</v>
       </c>
-      <c r="D60" s="21" t="s">
+      <c r="E60" s="21" t="s">
         <v>303</v>
       </c>
-      <c r="E60" s="21" t="s">
-        <v>304</v>
-      </c>
       <c r="F60" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H60" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I60" s="21"/>
       <c r="J60" s="21" t="str">
@@ -5202,25 +5562,25 @@
         <v>25</v>
       </c>
       <c r="B61" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="C61" s="21" t="s">
         <v>305</v>
       </c>
-      <c r="C61" s="21" t="s">
+      <c r="D61" s="21" t="s">
         <v>306</v>
       </c>
-      <c r="D61" s="21" t="s">
+      <c r="E61" s="21" t="s">
         <v>307</v>
-      </c>
-      <c r="E61" s="21" t="s">
-        <v>308</v>
       </c>
       <c r="F61" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G61" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H61" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I61" s="21"/>
       <c r="J61" s="21" t="str">
@@ -5240,25 +5600,25 @@
         <v>25</v>
       </c>
       <c r="B62" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="C62" s="21" t="s">
         <v>309</v>
       </c>
-      <c r="C62" s="21" t="s">
+      <c r="D62" s="21" t="s">
         <v>310</v>
       </c>
-      <c r="D62" s="21" t="s">
+      <c r="E62" s="21" t="s">
         <v>311</v>
-      </c>
-      <c r="E62" s="21" t="s">
-        <v>312</v>
       </c>
       <c r="F62" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G62" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H62" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I62" s="21"/>
       <c r="J62" s="21" t="str">
@@ -5278,25 +5638,25 @@
         <v>25</v>
       </c>
       <c r="B63" s="21" t="s">
+        <v>312</v>
+      </c>
+      <c r="C63" s="21" t="s">
         <v>313</v>
       </c>
-      <c r="C63" s="21" t="s">
+      <c r="D63" s="21" t="s">
         <v>314</v>
       </c>
-      <c r="D63" s="21" t="s">
+      <c r="E63" s="21" t="s">
         <v>315</v>
       </c>
-      <c r="E63" s="21" t="s">
-        <v>316</v>
-      </c>
       <c r="F63" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G63" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H63" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I63" s="21"/>
       <c r="J63" s="21" t="str">
@@ -5316,25 +5676,25 @@
         <v>25</v>
       </c>
       <c r="B64" s="21" t="s">
+        <v>316</v>
+      </c>
+      <c r="C64" s="21" t="s">
         <v>317</v>
       </c>
-      <c r="C64" s="21" t="s">
+      <c r="D64" s="21" t="s">
         <v>318</v>
       </c>
-      <c r="D64" s="21" t="s">
-        <v>319</v>
-      </c>
       <c r="E64" s="21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F64" s="21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G64" s="21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H64" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I64" s="21"/>
       <c r="J64" s="21" t="str">
@@ -5354,25 +5714,25 @@
         <v>25</v>
       </c>
       <c r="B65" s="21" t="s">
+        <v>319</v>
+      </c>
+      <c r="C65" s="21" t="s">
         <v>320</v>
       </c>
-      <c r="C65" s="21" t="s">
+      <c r="D65" s="21" t="s">
         <v>321</v>
       </c>
-      <c r="D65" s="21" t="s">
+      <c r="E65" s="21" t="s">
         <v>322</v>
-      </c>
-      <c r="E65" s="21" t="s">
-        <v>323</v>
       </c>
       <c r="F65" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G65" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H65" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I65" s="21"/>
       <c r="J65" s="21" t="str">
@@ -5392,25 +5752,25 @@
         <v>25</v>
       </c>
       <c r="B66" s="21" t="s">
+        <v>323</v>
+      </c>
+      <c r="C66" s="21" t="s">
         <v>324</v>
       </c>
-      <c r="C66" s="21" t="s">
+      <c r="D66" s="21" t="s">
         <v>325</v>
       </c>
-      <c r="D66" s="21" t="s">
+      <c r="E66" s="21" t="s">
         <v>326</v>
-      </c>
-      <c r="E66" s="21" t="s">
-        <v>327</v>
       </c>
       <c r="F66" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G66" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H66" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I66" s="21"/>
       <c r="J66" s="21" t="str">
@@ -5430,25 +5790,25 @@
         <v>25</v>
       </c>
       <c r="B67" s="21" t="s">
+        <v>327</v>
+      </c>
+      <c r="C67" s="21" t="s">
         <v>328</v>
       </c>
-      <c r="C67" s="21" t="s">
+      <c r="D67" s="21" t="s">
         <v>329</v>
       </c>
-      <c r="D67" s="21" t="s">
+      <c r="E67" s="21" t="s">
         <v>330</v>
-      </c>
-      <c r="E67" s="21" t="s">
-        <v>331</v>
       </c>
       <c r="F67" s="21" t="s">
         <v>78</v>
       </c>
       <c r="G67" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H67" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I67" s="21"/>
       <c r="J67" s="21" t="str">
@@ -5468,25 +5828,25 @@
         <v>26</v>
       </c>
       <c r="B68" s="21" t="s">
+        <v>331</v>
+      </c>
+      <c r="C68" s="21" t="s">
         <v>332</v>
       </c>
-      <c r="C68" s="21" t="s">
+      <c r="D68" s="21" t="s">
         <v>333</v>
       </c>
-      <c r="D68" s="21" t="s">
+      <c r="E68" s="21" t="s">
         <v>334</v>
-      </c>
-      <c r="E68" s="21" t="s">
-        <v>335</v>
       </c>
       <c r="F68" s="21" t="s">
         <v>78</v>
       </c>
       <c r="G68" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H68" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I68" s="21"/>
       <c r="J68" s="21" t="str">
@@ -5506,25 +5866,25 @@
         <v>26</v>
       </c>
       <c r="B69" s="21" t="s">
+        <v>335</v>
+      </c>
+      <c r="C69" s="21" t="s">
         <v>336</v>
       </c>
-      <c r="C69" s="21" t="s">
+      <c r="D69" s="21" t="s">
         <v>337</v>
       </c>
-      <c r="D69" s="21" t="s">
+      <c r="E69" s="21" t="s">
         <v>338</v>
-      </c>
-      <c r="E69" s="21" t="s">
-        <v>339</v>
       </c>
       <c r="F69" s="21" t="s">
         <v>78</v>
       </c>
       <c r="G69" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H69" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I69" s="21"/>
       <c r="J69" s="21" t="str">
@@ -5544,25 +5904,25 @@
         <v>26</v>
       </c>
       <c r="B70" s="21" t="s">
+        <v>339</v>
+      </c>
+      <c r="C70" s="21" t="s">
         <v>340</v>
       </c>
-      <c r="C70" s="21" t="s">
+      <c r="D70" s="21" t="s">
         <v>341</v>
       </c>
-      <c r="D70" s="21" t="s">
+      <c r="E70" s="21" t="s">
         <v>342</v>
-      </c>
-      <c r="E70" s="21" t="s">
-        <v>343</v>
       </c>
       <c r="F70" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G70" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H70" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I70" s="21"/>
       <c r="J70" s="21" t="str">
@@ -5582,25 +5942,25 @@
         <v>26</v>
       </c>
       <c r="B71" s="21" t="s">
+        <v>343</v>
+      </c>
+      <c r="C71" s="21" t="s">
         <v>344</v>
       </c>
-      <c r="C71" s="21" t="s">
+      <c r="D71" s="21" t="s">
         <v>345</v>
       </c>
-      <c r="D71" s="21" t="s">
+      <c r="E71" s="21" t="s">
         <v>346</v>
-      </c>
-      <c r="E71" s="21" t="s">
-        <v>347</v>
       </c>
       <c r="F71" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G71" s="21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H71" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I71" s="21"/>
       <c r="J71" s="21" t="str">
@@ -5620,25 +5980,25 @@
         <v>26</v>
       </c>
       <c r="B72" s="21" t="s">
+        <v>347</v>
+      </c>
+      <c r="C72" s="21" t="s">
         <v>348</v>
       </c>
-      <c r="C72" s="21" t="s">
+      <c r="D72" s="21" t="s">
         <v>349</v>
       </c>
-      <c r="D72" s="21" t="s">
+      <c r="E72" s="21" t="s">
         <v>350</v>
-      </c>
-      <c r="E72" s="21" t="s">
-        <v>351</v>
       </c>
       <c r="F72" s="21" t="s">
         <v>78</v>
       </c>
       <c r="G72" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H72" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I72" s="21"/>
       <c r="J72" s="21" t="str">
@@ -5658,25 +6018,25 @@
         <v>26</v>
       </c>
       <c r="B73" s="21" t="s">
+        <v>351</v>
+      </c>
+      <c r="C73" s="21" t="s">
         <v>352</v>
       </c>
-      <c r="C73" s="21" t="s">
+      <c r="D73" s="21" t="s">
         <v>353</v>
       </c>
-      <c r="D73" s="21" t="s">
+      <c r="E73" s="21" t="s">
         <v>354</v>
-      </c>
-      <c r="E73" s="21" t="s">
-        <v>355</v>
       </c>
       <c r="F73" s="21" t="s">
         <v>38</v>
       </c>
       <c r="G73" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H73" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I73" s="21"/>
       <c r="J73" s="21" t="str">
@@ -5696,25 +6056,25 @@
         <v>26</v>
       </c>
       <c r="B74" s="21" t="s">
+        <v>355</v>
+      </c>
+      <c r="C74" s="21" t="s">
         <v>356</v>
       </c>
-      <c r="C74" s="21" t="s">
+      <c r="D74" s="21" t="s">
         <v>357</v>
       </c>
-      <c r="D74" s="21" t="s">
+      <c r="E74" s="21" t="s">
         <v>358</v>
-      </c>
-      <c r="E74" s="21" t="s">
-        <v>359</v>
       </c>
       <c r="F74" s="21" t="s">
         <v>34</v>
       </c>
       <c r="G74" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H74" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I74" s="21"/>
       <c r="J74" s="21" t="str">
@@ -5734,25 +6094,25 @@
         <v>26</v>
       </c>
       <c r="B75" s="21" t="s">
+        <v>359</v>
+      </c>
+      <c r="C75" s="21" t="s">
         <v>360</v>
       </c>
-      <c r="C75" s="21" t="s">
+      <c r="D75" s="21" t="s">
         <v>361</v>
       </c>
-      <c r="D75" s="21" t="s">
+      <c r="E75" s="21" t="s">
         <v>362</v>
-      </c>
-      <c r="E75" s="21" t="s">
-        <v>363</v>
       </c>
       <c r="F75" s="21" t="s">
         <v>81</v>
       </c>
       <c r="G75" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H75" s="21" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I75" s="21"/>
       <c r="J75" s="21" t="str">
@@ -5772,25 +6132,25 @@
         <v>26</v>
       </c>
       <c r="B76" s="22" t="s">
+        <v>363</v>
+      </c>
+      <c r="C76" s="22" t="s">
         <v>364</v>
       </c>
-      <c r="C76" s="22" t="s">
+      <c r="D76" s="22" t="s">
         <v>365</v>
       </c>
-      <c r="D76" s="22" t="s">
+      <c r="E76" s="22" t="s">
         <v>366</v>
-      </c>
-      <c r="E76" s="22" t="s">
-        <v>367</v>
       </c>
       <c r="F76" s="22" t="s">
         <v>38</v>
       </c>
       <c r="G76" s="22" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H76" s="22" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="I76" s="22"/>
       <c r="J76" s="22" t="str">
@@ -5807,17 +6167,6 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="C1:Q1"/>
-    <mergeCell ref="C2:Q2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="M3:Q3"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="I4:L4"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="A6:Q6"/>
     <mergeCell ref="A10:Q10"/>
     <mergeCell ref="P7:Q7"/>
     <mergeCell ref="A8:B9"/>
@@ -5831,6 +6180,17 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="I4:L4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="A6:Q6"/>
+    <mergeCell ref="C1:Q1"/>
+    <mergeCell ref="C2:Q2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:Q3"/>
   </mergeCells>
   <conditionalFormatting sqref="G13:G76">
     <cfRule type="cellIs" dxfId="12" priority="5" operator="equal">
@@ -5863,6 +6223,13 @@
       </dataBar>
     </cfRule>
     <cfRule type="dataBar" priority="15">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFC92351"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -5907,40 +6274,6 @@
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000000000000}">
-          <x14:formula1>
-            <xm:f>Catálogos!$E$2:$E$8</xm:f>
-          </x14:formula1>
-          <xm:sqref>F13:F76 O13:O76</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000001000000}">
-          <x14:formula1>
-            <xm:f>Catálogos!$A$2:$A$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>G13:G76</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000002000000}">
-          <x14:formula1>
-            <xm:f>Catálogos!$B$2:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>H13:H76</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000003000000}">
-          <x14:formula1>
-            <xm:f>Catálogos!$C$2:$C$5</xm:f>
-          </x14:formula1>
-          <xm:sqref>I13:I76</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0100-000005000000}">
-          <x14:formula1>
-            <xm:f>Catálogos!$D$2:$D$6</xm:f>
-          </x14:formula1>
-          <xm:sqref>Q13:Q76</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
   </extLst>
 </worksheet>
 </file>
@@ -5959,76 +6292,76 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>368</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C2" s="7" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>78</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>371</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>372</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>373</v>
-      </c>
       <c r="D3" s="7" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>38</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>375</v>
+        <v>111</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>9</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>81</v>
@@ -6037,17 +6370,17 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="6" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F5" s="8"/>
     </row>
@@ -6056,10 +6389,10 @@
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F6" s="8"/>
     </row>
@@ -6079,11 +6412,487 @@
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="F8" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <tabColor rgb="FF2A3966"/>
+  </sheetPr>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.796875" defaultRowHeight="13.8"/>
+  <cols>
+    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="2" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="32" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.05" customHeight="1">
+      <c r="A1" s="67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+    </row>
+    <row r="2" spans="1:8" ht="25.95" customHeight="1">
+      <c r="A2" s="67" t="s">
+        <v>385</v>
+      </c>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="67"/>
+      <c r="F2" s="67"/>
+      <c r="G2" s="67"/>
+      <c r="H2" s="67"/>
+    </row>
+    <row r="3" spans="1:8" ht="22.05" customHeight="1">
+      <c r="A3" s="68" t="s">
+        <v>386</v>
+      </c>
+      <c r="B3" s="68"/>
+      <c r="C3" s="68"/>
+      <c r="D3" s="68"/>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="68"/>
+      <c r="H3" s="68"/>
+    </row>
+    <row r="5" spans="1:8" ht="37.950000000000003" customHeight="1">
+      <c r="A5" s="69" t="s">
+        <v>387</v>
+      </c>
+      <c r="B5" s="69"/>
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="69"/>
+      <c r="G5" s="69"/>
+      <c r="H5" s="69"/>
+    </row>
+    <row r="7" spans="1:8" ht="34.049999999999997" customHeight="1">
+      <c r="A7" s="39" t="s">
+        <v>388</v>
+      </c>
+      <c r="B7" s="70" t="s">
+        <v>389</v>
+      </c>
+      <c r="C7" s="70"/>
+      <c r="D7" s="39" t="s">
+        <v>390</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>391</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>392</v>
+      </c>
+      <c r="G7" s="39" t="s">
+        <v>393</v>
+      </c>
+      <c r="H7" s="39" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="54" customHeight="1">
+      <c r="A8" s="41">
+        <v>1</v>
+      </c>
+      <c r="B8" s="71" t="s">
+        <v>395</v>
+      </c>
+      <c r="C8" s="71"/>
+      <c r="D8" s="40" t="s">
+        <v>396</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>397</v>
+      </c>
+      <c r="F8" s="41" t="s">
+        <v>398</v>
+      </c>
+      <c r="G8" s="40" t="s">
+        <v>399</v>
+      </c>
+      <c r="H8" s="40" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="54" customHeight="1">
+      <c r="A9" s="43">
+        <v>2</v>
+      </c>
+      <c r="B9" s="72" t="s">
+        <v>401</v>
+      </c>
+      <c r="C9" s="72"/>
+      <c r="D9" s="42" t="s">
+        <v>402</v>
+      </c>
+      <c r="E9" s="42" t="s">
+        <v>403</v>
+      </c>
+      <c r="F9" s="43" t="s">
+        <v>404</v>
+      </c>
+      <c r="G9" s="42" t="s">
+        <v>405</v>
+      </c>
+      <c r="H9" s="42" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="54" customHeight="1">
+      <c r="A10" s="41">
+        <v>3</v>
+      </c>
+      <c r="B10" s="71" t="s">
+        <v>407</v>
+      </c>
+      <c r="C10" s="71"/>
+      <c r="D10" s="40" t="s">
+        <v>408</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>409</v>
+      </c>
+      <c r="F10" s="41" t="s">
+        <v>410</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>411</v>
+      </c>
+      <c r="H10" s="40" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="54" customHeight="1">
+      <c r="A11" s="43">
+        <v>4</v>
+      </c>
+      <c r="B11" s="72" t="s">
+        <v>413</v>
+      </c>
+      <c r="C11" s="72"/>
+      <c r="D11" s="42" t="s">
+        <v>414</v>
+      </c>
+      <c r="E11" s="42" t="s">
+        <v>415</v>
+      </c>
+      <c r="F11" s="43" t="s">
+        <v>416</v>
+      </c>
+      <c r="G11" s="42" t="s">
+        <v>417</v>
+      </c>
+      <c r="H11" s="42" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="54" customHeight="1">
+      <c r="A12" s="41">
+        <v>5</v>
+      </c>
+      <c r="B12" s="71" t="s">
+        <v>419</v>
+      </c>
+      <c r="C12" s="71"/>
+      <c r="D12" s="40" t="s">
+        <v>420</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>421</v>
+      </c>
+      <c r="F12" s="41" t="s">
+        <v>422</v>
+      </c>
+      <c r="G12" s="40" t="s">
+        <v>423</v>
+      </c>
+      <c r="H12" s="40" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="54" customHeight="1">
+      <c r="A13" s="43">
+        <v>6</v>
+      </c>
+      <c r="B13" s="72" t="s">
+        <v>425</v>
+      </c>
+      <c r="C13" s="72"/>
+      <c r="D13" s="42" t="s">
+        <v>426</v>
+      </c>
+      <c r="E13" s="42" t="s">
+        <v>427</v>
+      </c>
+      <c r="F13" s="43" t="s">
+        <v>428</v>
+      </c>
+      <c r="G13" s="42" t="s">
+        <v>429</v>
+      </c>
+      <c r="H13" s="42" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="54" customHeight="1">
+      <c r="A14" s="41">
+        <v>7</v>
+      </c>
+      <c r="B14" s="71" t="s">
+        <v>431</v>
+      </c>
+      <c r="C14" s="71"/>
+      <c r="D14" s="40" t="s">
+        <v>432</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>433</v>
+      </c>
+      <c r="F14" s="41" t="s">
+        <v>434</v>
+      </c>
+      <c r="G14" s="40" t="s">
+        <v>435</v>
+      </c>
+      <c r="H14" s="40" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="54" customHeight="1">
+      <c r="A15" s="43">
+        <v>8</v>
+      </c>
+      <c r="B15" s="72" t="s">
+        <v>437</v>
+      </c>
+      <c r="C15" s="72"/>
+      <c r="D15" s="42" t="s">
+        <v>438</v>
+      </c>
+      <c r="E15" s="42" t="s">
+        <v>439</v>
+      </c>
+      <c r="F15" s="43" t="s">
+        <v>410</v>
+      </c>
+      <c r="G15" s="42" t="s">
+        <v>440</v>
+      </c>
+      <c r="H15" s="42" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="54" customHeight="1">
+      <c r="A16" s="41">
+        <v>9</v>
+      </c>
+      <c r="B16" s="71" t="s">
+        <v>442</v>
+      </c>
+      <c r="C16" s="71"/>
+      <c r="D16" s="40" t="s">
+        <v>443</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>444</v>
+      </c>
+      <c r="F16" s="41" t="s">
+        <v>445</v>
+      </c>
+      <c r="G16" s="40" t="s">
+        <v>446</v>
+      </c>
+      <c r="H16" s="40" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="54" customHeight="1">
+      <c r="A17" s="43">
+        <v>10</v>
+      </c>
+      <c r="B17" s="72" t="s">
+        <v>448</v>
+      </c>
+      <c r="C17" s="72"/>
+      <c r="D17" s="42" t="s">
+        <v>449</v>
+      </c>
+      <c r="E17" s="42" t="s">
+        <v>450</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>451</v>
+      </c>
+      <c r="G17" s="42" t="s">
+        <v>452</v>
+      </c>
+      <c r="H17" s="42" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="54" customHeight="1">
+      <c r="A18" s="41">
+        <v>11</v>
+      </c>
+      <c r="B18" s="71" t="s">
+        <v>454</v>
+      </c>
+      <c r="C18" s="71"/>
+      <c r="D18" s="40" t="s">
+        <v>455</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>456</v>
+      </c>
+      <c r="F18" s="41" t="s">
+        <v>457</v>
+      </c>
+      <c r="G18" s="40" t="s">
+        <v>458</v>
+      </c>
+      <c r="H18" s="40" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="54" customHeight="1">
+      <c r="A19" s="43">
+        <v>12</v>
+      </c>
+      <c r="B19" s="72" t="s">
+        <v>460</v>
+      </c>
+      <c r="C19" s="72"/>
+      <c r="D19" s="42" t="s">
+        <v>461</v>
+      </c>
+      <c r="E19" s="42" t="s">
+        <v>462</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>463</v>
+      </c>
+      <c r="G19" s="42" t="s">
+        <v>464</v>
+      </c>
+      <c r="H19" s="42" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="54" customHeight="1">
+      <c r="A20" s="41">
+        <v>13</v>
+      </c>
+      <c r="B20" s="71" t="s">
+        <v>466</v>
+      </c>
+      <c r="C20" s="71"/>
+      <c r="D20" s="40" t="s">
+        <v>467</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>468</v>
+      </c>
+      <c r="F20" s="41" t="s">
+        <v>451</v>
+      </c>
+      <c r="G20" s="40" t="s">
+        <v>469</v>
+      </c>
+      <c r="H20" s="40" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="54" customHeight="1">
+      <c r="A21" s="43">
+        <v>14</v>
+      </c>
+      <c r="B21" s="72" t="s">
+        <v>471</v>
+      </c>
+      <c r="C21" s="72"/>
+      <c r="D21" s="42" t="s">
+        <v>472</v>
+      </c>
+      <c r="E21" s="42" t="s">
+        <v>473</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>474</v>
+      </c>
+      <c r="G21" s="42" t="s">
+        <v>475</v>
+      </c>
+      <c r="H21" s="42" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="54" customHeight="1">
+      <c r="A22" s="41">
+        <v>15</v>
+      </c>
+      <c r="B22" s="71" t="s">
+        <v>476</v>
+      </c>
+      <c r="C22" s="71"/>
+      <c r="D22" s="40" t="s">
+        <v>477</v>
+      </c>
+      <c r="E22" s="40" t="s">
+        <v>478</v>
+      </c>
+      <c r="F22" s="41" t="s">
+        <v>463</v>
+      </c>
+      <c r="G22" s="40" t="s">
+        <v>479</v>
+      </c>
+      <c r="H22" s="40" t="s">
+        <v>480</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizaicon del doucmento de Vision
</commit_message>
<xml_diff>
--- a/Documentacion/12 Matriz de Gestion de Calidad.xlsx
+++ b/Documentacion/12 Matriz de Gestion de Calidad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexMendoza\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\U Alex\Ingenieria Software 2\Proyecto Ingenieria II\Documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CCD307D-9169-497F-A23E-64F55BC33354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="735" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -2053,6 +2053,24 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2061,34 +2079,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2116,23 +2110,29 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2663,35 +2663,35 @@
   <sheetData>
     <row r="1" spans="1:12" ht="24" customHeight="1">
       <c r="A1" s="1"/>
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="50" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51"/>
+      <c r="G1" s="51"/>
+      <c r="H1" s="51"/>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
+      <c r="K1" s="51"/>
+      <c r="L1" s="51"/>
     </row>
     <row r="2" spans="1:12" ht="24" customHeight="1">
       <c r="A2" s="12"/>
-      <c r="B2" s="46" t="s">
+      <c r="B2" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-      <c r="F2" s="47"/>
-      <c r="G2" s="47"/>
-      <c r="H2" s="47"/>
-      <c r="I2" s="47"/>
-      <c r="J2" s="47"/>
-      <c r="K2" s="47"/>
-      <c r="L2" s="47"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="53"/>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="I2" s="53"/>
+      <c r="J2" s="53"/>
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
     </row>
     <row r="3" spans="1:12" ht="24" customHeight="1">
       <c r="A3" s="13"/>
@@ -3435,98 +3435,98 @@
     <row r="1" spans="1:17" ht="25.05" customHeight="1">
       <c r="A1" s="12"/>
       <c r="B1" s="12"/>
-      <c r="C1" s="48" t="s">
+      <c r="C1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="47"/>
-      <c r="L1" s="47"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="47"/>
-      <c r="P1" s="47"/>
-      <c r="Q1" s="47"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="53"/>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
     </row>
     <row r="2" spans="1:17" ht="25.05" customHeight="1">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
-      <c r="C2" s="46" t="s">
+      <c r="C2" s="52" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
-      <c r="H2" s="49"/>
-      <c r="I2" s="49"/>
-      <c r="J2" s="49"/>
-      <c r="K2" s="49"/>
-      <c r="L2" s="49"/>
-      <c r="M2" s="49"/>
-      <c r="N2" s="49"/>
-      <c r="O2" s="49"/>
-      <c r="P2" s="49"/>
-      <c r="Q2" s="49"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="55"/>
+      <c r="J2" s="55"/>
+      <c r="K2" s="55"/>
+      <c r="L2" s="55"/>
+      <c r="M2" s="55"/>
+      <c r="N2" s="55"/>
+      <c r="O2" s="55"/>
+      <c r="P2" s="55"/>
+      <c r="Q2" s="55"/>
     </row>
     <row r="3" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A3" s="50" t="s">
+      <c r="A3" s="70" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="51"/>
-      <c r="C3" s="51"/>
-      <c r="D3" s="51"/>
-      <c r="E3" s="51" t="s">
+      <c r="B3" s="71"/>
+      <c r="C3" s="71"/>
+      <c r="D3" s="71"/>
+      <c r="E3" s="71" t="s">
         <v>383</v>
       </c>
-      <c r="F3" s="51"/>
-      <c r="G3" s="51"/>
-      <c r="H3" s="51"/>
-      <c r="I3" s="51" t="s">
+      <c r="F3" s="71"/>
+      <c r="G3" s="71"/>
+      <c r="H3" s="71"/>
+      <c r="I3" s="71" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="51"/>
-      <c r="K3" s="51"/>
-      <c r="L3" s="51" t="s">
+      <c r="J3" s="71"/>
+      <c r="K3" s="71"/>
+      <c r="L3" s="71" t="s">
         <v>384</v>
       </c>
-      <c r="M3" s="51"/>
-      <c r="N3" s="51"/>
-      <c r="O3" s="51"/>
-      <c r="P3" s="51"/>
-      <c r="Q3" s="52"/>
+      <c r="M3" s="71"/>
+      <c r="N3" s="71"/>
+      <c r="O3" s="71"/>
+      <c r="P3" s="71"/>
+      <c r="Q3" s="72"/>
     </row>
     <row r="4" spans="1:17" ht="22.05" customHeight="1">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="65" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54" t="s">
+      <c r="B4" s="66"/>
+      <c r="C4" s="66"/>
+      <c r="D4" s="66"/>
+      <c r="E4" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54" t="s">
+      <c r="F4" s="66"/>
+      <c r="G4" s="66"/>
+      <c r="H4" s="66"/>
+      <c r="I4" s="66" t="s">
         <v>86</v>
       </c>
-      <c r="J4" s="54"/>
-      <c r="K4" s="54"/>
-      <c r="L4" s="54"/>
-      <c r="M4" s="54" t="s">
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66" t="s">
         <v>87</v>
       </c>
-      <c r="N4" s="54"/>
-      <c r="O4" s="54"/>
-      <c r="P4" s="54"/>
-      <c r="Q4" s="55"/>
+      <c r="N4" s="66"/>
+      <c r="O4" s="66"/>
+      <c r="P4" s="66"/>
+      <c r="Q4" s="67"/>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="13"/>
@@ -3548,133 +3548,133 @@
       <c r="Q5" s="13"/>
     </row>
     <row r="6" spans="1:17" ht="24" customHeight="1">
-      <c r="A6" s="56" t="s">
+      <c r="A6" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="49"/>
-      <c r="I6" s="49"/>
-      <c r="J6" s="49"/>
-      <c r="K6" s="49"/>
-      <c r="L6" s="49"/>
-      <c r="M6" s="49"/>
-      <c r="N6" s="49"/>
-      <c r="O6" s="49"/>
-      <c r="P6" s="49"/>
-      <c r="Q6" s="49"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
+      <c r="J6" s="55"/>
+      <c r="K6" s="55"/>
+      <c r="L6" s="55"/>
+      <c r="M6" s="55"/>
+      <c r="N6" s="55"/>
+      <c r="O6" s="55"/>
+      <c r="P6" s="55"/>
+      <c r="Q6" s="55"/>
     </row>
     <row r="7" spans="1:17" ht="24" customHeight="1">
-      <c r="A7" s="58" t="s">
+      <c r="A7" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="58"/>
+      <c r="B7" s="56"/>
       <c r="C7" s="14"/>
-      <c r="D7" s="58" t="s">
+      <c r="D7" s="56" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="58"/>
+      <c r="E7" s="56"/>
       <c r="F7" s="14"/>
-      <c r="G7" s="58" t="s">
+      <c r="G7" s="56" t="s">
         <v>15</v>
       </c>
-      <c r="H7" s="58"/>
+      <c r="H7" s="56"/>
       <c r="I7" s="14"/>
-      <c r="J7" s="58" t="s">
+      <c r="J7" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="K7" s="58"/>
+      <c r="K7" s="56"/>
       <c r="L7" s="14"/>
-      <c r="M7" s="58" t="s">
+      <c r="M7" s="56" t="s">
         <v>89</v>
       </c>
-      <c r="N7" s="58"/>
+      <c r="N7" s="56"/>
       <c r="O7" s="14"/>
-      <c r="P7" s="58" t="s">
+      <c r="P7" s="56" t="s">
         <v>23</v>
       </c>
-      <c r="Q7" s="58"/>
+      <c r="Q7" s="56"/>
     </row>
     <row r="8" spans="1:17" ht="24" customHeight="1">
-      <c r="A8" s="59">
+      <c r="A8" s="57">
         <f>COUNTA(A13:A76)</f>
         <v>64</v>
       </c>
-      <c r="B8" s="60"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="15"/>
-      <c r="D8" s="60">
+      <c r="D8" s="58">
         <f>COUNTIF(I13:I76,"Cumple")+COUNTIF(I13:I76,"Cumple parcialmente")+COUNTIF(I13:I76,"No cumple")+COUNTIF(I13:I76,"No aplica")</f>
         <v>2</v>
       </c>
-      <c r="E8" s="60"/>
+      <c r="E8" s="58"/>
       <c r="F8" s="15"/>
-      <c r="G8" s="63">
+      <c r="G8" s="61">
         <f>IFERROR(D8/A8,0)</f>
         <v>3.125E-2</v>
       </c>
-      <c r="H8" s="63"/>
+      <c r="H8" s="61"/>
       <c r="I8" s="15"/>
-      <c r="J8" s="63">
+      <c r="J8" s="61">
         <f>IFERROR(SUM(J13:J76)/(COUNT(J13:J76)*2),0)</f>
         <v>1</v>
       </c>
-      <c r="K8" s="63"/>
+      <c r="K8" s="61"/>
       <c r="L8" s="15"/>
-      <c r="M8" s="63">
+      <c r="M8" s="61">
         <f>IFERROR(COUNTIF(I13:I76,"Cumple")/COUNT(J13:J76),0)</f>
         <v>1</v>
       </c>
-      <c r="N8" s="63"/>
+      <c r="N8" s="61"/>
       <c r="O8" s="15"/>
-      <c r="P8" s="60" t="str">
+      <c r="P8" s="58" t="str">
         <f>IF(G8&lt;1,"PENDIENTE DE EVALUACIÓN",IF(COUNTIFS(G13:G76,"Highest",I13:I76,"No cumple")&gt;0,"NO APROBADO",IF(J8&gt;=0.9,"APROBADO","REQUIERE MEJORAS")))</f>
         <v>PENDIENTE DE EVALUACIÓN</v>
       </c>
-      <c r="Q8" s="65"/>
+      <c r="Q8" s="63"/>
     </row>
     <row r="9" spans="1:17" ht="24" customHeight="1">
-      <c r="A9" s="61"/>
-      <c r="B9" s="62"/>
+      <c r="A9" s="59"/>
+      <c r="B9" s="60"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
+      <c r="D9" s="60"/>
+      <c r="E9" s="60"/>
       <c r="F9" s="16"/>
-      <c r="G9" s="64"/>
-      <c r="H9" s="64"/>
+      <c r="G9" s="62"/>
+      <c r="H9" s="62"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="64"/>
-      <c r="K9" s="64"/>
+      <c r="J9" s="62"/>
+      <c r="K9" s="62"/>
       <c r="L9" s="16"/>
-      <c r="M9" s="64"/>
-      <c r="N9" s="64"/>
+      <c r="M9" s="62"/>
+      <c r="N9" s="62"/>
       <c r="O9" s="16"/>
-      <c r="P9" s="62"/>
-      <c r="Q9" s="66"/>
+      <c r="P9" s="60"/>
+      <c r="Q9" s="64"/>
     </row>
     <row r="10" spans="1:17" ht="24" customHeight="1">
-      <c r="A10" s="57" t="s">
+      <c r="A10" s="54" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="49"/>
-      <c r="C10" s="49"/>
-      <c r="D10" s="49"/>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
-      <c r="G10" s="49"/>
-      <c r="H10" s="49"/>
-      <c r="I10" s="49"/>
-      <c r="J10" s="49"/>
-      <c r="K10" s="49"/>
-      <c r="L10" s="49"/>
-      <c r="M10" s="49"/>
-      <c r="N10" s="49"/>
-      <c r="O10" s="49"/>
-      <c r="P10" s="49"/>
-      <c r="Q10" s="49"/>
+      <c r="B10" s="55"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="55"/>
+      <c r="N10" s="55"/>
+      <c r="O10" s="55"/>
+      <c r="P10" s="55"/>
+      <c r="Q10" s="55"/>
     </row>
     <row r="12" spans="1:17" ht="42" customHeight="1">
       <c r="A12" s="17" t="s">
@@ -6167,6 +6167,17 @@
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C1:Q1"/>
+    <mergeCell ref="C2:Q2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:H3"/>
+    <mergeCell ref="I3:L3"/>
+    <mergeCell ref="M3:Q3"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="I4:L4"/>
+    <mergeCell ref="M4:Q4"/>
+    <mergeCell ref="A6:Q6"/>
     <mergeCell ref="A10:Q10"/>
     <mergeCell ref="P7:Q7"/>
     <mergeCell ref="A8:B9"/>
@@ -6180,17 +6191,6 @@
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="I4:L4"/>
-    <mergeCell ref="M4:Q4"/>
-    <mergeCell ref="A6:Q6"/>
-    <mergeCell ref="C1:Q1"/>
-    <mergeCell ref="C2:Q2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:H3"/>
-    <mergeCell ref="I3:L3"/>
-    <mergeCell ref="M3:Q3"/>
   </mergeCells>
   <conditionalFormatting sqref="G13:G76">
     <cfRule type="cellIs" dxfId="12" priority="5" operator="equal">
@@ -6439,61 +6439,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="28.05" customHeight="1">
-      <c r="A1" s="67" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
     </row>
     <row r="2" spans="1:8" ht="25.95" customHeight="1">
-      <c r="A2" s="67" t="s">
+      <c r="A2" s="46" t="s">
         <v>385</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="67"/>
-      <c r="F2" s="67"/>
-      <c r="G2" s="67"/>
-      <c r="H2" s="67"/>
+      <c r="B2" s="46"/>
+      <c r="C2" s="46"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
     </row>
     <row r="3" spans="1:8" ht="22.05" customHeight="1">
-      <c r="A3" s="68" t="s">
+      <c r="A3" s="47" t="s">
         <v>386</v>
       </c>
-      <c r="B3" s="68"/>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="F3" s="68"/>
-      <c r="G3" s="68"/>
-      <c r="H3" s="68"/>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
     </row>
     <row r="5" spans="1:8" ht="37.950000000000003" customHeight="1">
-      <c r="A5" s="69" t="s">
+      <c r="A5" s="48" t="s">
         <v>387</v>
       </c>
-      <c r="B5" s="69"/>
-      <c r="C5" s="69"/>
-      <c r="D5" s="69"/>
-      <c r="E5" s="69"/>
-      <c r="F5" s="69"/>
-      <c r="G5" s="69"/>
-      <c r="H5" s="69"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="48"/>
     </row>
     <row r="7" spans="1:8" ht="34.049999999999997" customHeight="1">
       <c r="A7" s="39" t="s">
         <v>388</v>
       </c>
-      <c r="B7" s="70" t="s">
+      <c r="B7" s="49" t="s">
         <v>389</v>
       </c>
-      <c r="C7" s="70"/>
+      <c r="C7" s="49"/>
       <c r="D7" s="39" t="s">
         <v>390</v>
       </c>
@@ -6514,10 +6514,10 @@
       <c r="A8" s="41">
         <v>1</v>
       </c>
-      <c r="B8" s="71" t="s">
+      <c r="B8" s="44" t="s">
         <v>395</v>
       </c>
-      <c r="C8" s="71"/>
+      <c r="C8" s="44"/>
       <c r="D8" s="40" t="s">
         <v>396</v>
       </c>
@@ -6538,10 +6538,10 @@
       <c r="A9" s="43">
         <v>2</v>
       </c>
-      <c r="B9" s="72" t="s">
+      <c r="B9" s="45" t="s">
         <v>401</v>
       </c>
-      <c r="C9" s="72"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="42" t="s">
         <v>402</v>
       </c>
@@ -6562,10 +6562,10 @@
       <c r="A10" s="41">
         <v>3</v>
       </c>
-      <c r="B10" s="71" t="s">
+      <c r="B10" s="44" t="s">
         <v>407</v>
       </c>
-      <c r="C10" s="71"/>
+      <c r="C10" s="44"/>
       <c r="D10" s="40" t="s">
         <v>408</v>
       </c>
@@ -6586,10 +6586,10 @@
       <c r="A11" s="43">
         <v>4</v>
       </c>
-      <c r="B11" s="72" t="s">
+      <c r="B11" s="45" t="s">
         <v>413</v>
       </c>
-      <c r="C11" s="72"/>
+      <c r="C11" s="45"/>
       <c r="D11" s="42" t="s">
         <v>414</v>
       </c>
@@ -6610,10 +6610,10 @@
       <c r="A12" s="41">
         <v>5</v>
       </c>
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="44" t="s">
         <v>419</v>
       </c>
-      <c r="C12" s="71"/>
+      <c r="C12" s="44"/>
       <c r="D12" s="40" t="s">
         <v>420</v>
       </c>
@@ -6634,10 +6634,10 @@
       <c r="A13" s="43">
         <v>6</v>
       </c>
-      <c r="B13" s="72" t="s">
+      <c r="B13" s="45" t="s">
         <v>425</v>
       </c>
-      <c r="C13" s="72"/>
+      <c r="C13" s="45"/>
       <c r="D13" s="42" t="s">
         <v>426</v>
       </c>
@@ -6658,10 +6658,10 @@
       <c r="A14" s="41">
         <v>7</v>
       </c>
-      <c r="B14" s="71" t="s">
+      <c r="B14" s="44" t="s">
         <v>431</v>
       </c>
-      <c r="C14" s="71"/>
+      <c r="C14" s="44"/>
       <c r="D14" s="40" t="s">
         <v>432</v>
       </c>
@@ -6682,10 +6682,10 @@
       <c r="A15" s="43">
         <v>8</v>
       </c>
-      <c r="B15" s="72" t="s">
+      <c r="B15" s="45" t="s">
         <v>437</v>
       </c>
-      <c r="C15" s="72"/>
+      <c r="C15" s="45"/>
       <c r="D15" s="42" t="s">
         <v>438</v>
       </c>
@@ -6706,10 +6706,10 @@
       <c r="A16" s="41">
         <v>9</v>
       </c>
-      <c r="B16" s="71" t="s">
+      <c r="B16" s="44" t="s">
         <v>442</v>
       </c>
-      <c r="C16" s="71"/>
+      <c r="C16" s="44"/>
       <c r="D16" s="40" t="s">
         <v>443</v>
       </c>
@@ -6730,10 +6730,10 @@
       <c r="A17" s="43">
         <v>10</v>
       </c>
-      <c r="B17" s="72" t="s">
+      <c r="B17" s="45" t="s">
         <v>448</v>
       </c>
-      <c r="C17" s="72"/>
+      <c r="C17" s="45"/>
       <c r="D17" s="42" t="s">
         <v>449</v>
       </c>
@@ -6754,10 +6754,10 @@
       <c r="A18" s="41">
         <v>11</v>
       </c>
-      <c r="B18" s="71" t="s">
+      <c r="B18" s="44" t="s">
         <v>454</v>
       </c>
-      <c r="C18" s="71"/>
+      <c r="C18" s="44"/>
       <c r="D18" s="40" t="s">
         <v>455</v>
       </c>
@@ -6778,10 +6778,10 @@
       <c r="A19" s="43">
         <v>12</v>
       </c>
-      <c r="B19" s="72" t="s">
+      <c r="B19" s="45" t="s">
         <v>460</v>
       </c>
-      <c r="C19" s="72"/>
+      <c r="C19" s="45"/>
       <c r="D19" s="42" t="s">
         <v>461</v>
       </c>
@@ -6802,10 +6802,10 @@
       <c r="A20" s="41">
         <v>13</v>
       </c>
-      <c r="B20" s="71" t="s">
+      <c r="B20" s="44" t="s">
         <v>466</v>
       </c>
-      <c r="C20" s="71"/>
+      <c r="C20" s="44"/>
       <c r="D20" s="40" t="s">
         <v>467</v>
       </c>
@@ -6826,10 +6826,10 @@
       <c r="A21" s="43">
         <v>14</v>
       </c>
-      <c r="B21" s="72" t="s">
+      <c r="B21" s="45" t="s">
         <v>471</v>
       </c>
-      <c r="C21" s="72"/>
+      <c r="C21" s="45"/>
       <c r="D21" s="42" t="s">
         <v>472</v>
       </c>
@@ -6850,10 +6850,10 @@
       <c r="A22" s="41">
         <v>15</v>
       </c>
-      <c r="B22" s="71" t="s">
+      <c r="B22" s="44" t="s">
         <v>476</v>
       </c>
-      <c r="C22" s="71"/>
+      <c r="C22" s="44"/>
       <c r="D22" s="40" t="s">
         <v>477</v>
       </c>
@@ -6872,26 +6872,26 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B20:C20"/>
     <mergeCell ref="B21:C21"/>
     <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="B7:C7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>